<commit_message>
Update model, report and README
</commit_message>
<xml_diff>
--- a/Ryanair_DCF_Model_Kodickova_2026.xlsx
+++ b/Ryanair_DCF_Model_Kodickova_2026.xlsx
@@ -447,7 +447,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="301">
   <si>
     <t xml:space="preserve">DCF Model - Ryanair</t>
   </si>
@@ -810,24 +810,6 @@
   </si>
   <si>
     <t xml:space="preserve">Tolerance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Known weak points</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tax at 10% against Pillar Two. 15% would give about 28 per share on the original model and about 31.5 on the final model.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FY26 FCF is not prorated for the stub period.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The "Total Debt 10,470" label in the Ratios balance sheet table is actually total liabilities.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leases are not added to debt separately.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The RONIC path (19.1% in FY26 fading to WACC in FY35) is an analyst assumption.</t>
   </si>
   <si>
     <t xml:space="preserve">Comps</t>
@@ -7131,7 +7113,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:F48"/>
+  <dimension ref="B1:F41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
@@ -7708,40 +7690,6 @@
       </c>
       <c r="C41" s="103" t="n">
         <v>0.3</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B43" s="86" t="s">
-        <v>121</v>
-      </c>
-      <c r="C43" s="86"/>
-      <c r="D43" s="86"/>
-      <c r="E43" s="86"/>
-      <c r="F43" s="86"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B44" s="91" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B45" s="91" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B46" s="91" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B47" s="91" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B48" s="91" t="s">
-        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -7780,7 +7728,7 @@
   <sheetData>
     <row r="2" s="2" customFormat="true" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="104" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7797,7 +7745,7 @@
       <c r="L4" s="15"/>
       <c r="M4" s="15"/>
       <c r="N4" s="105" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="O4" s="105"/>
       <c r="P4" s="105"/>
@@ -7805,14 +7753,14 @@
       <c r="R4" s="105"/>
       <c r="S4" s="15"/>
       <c r="T4" s="105" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="U4" s="105"/>
       <c r="V4" s="105"/>
       <c r="W4" s="105"/>
       <c r="X4" s="105"/>
       <c r="Y4" s="106" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="Z4" s="106"/>
     </row>
@@ -7824,49 +7772,49 @@
       <c r="F5" s="34"/>
       <c r="G5" s="34"/>
       <c r="H5" s="107" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="I5" s="108"/>
       <c r="J5" s="107" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="K5" s="108"/>
       <c r="L5" s="107" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="M5" s="109"/>
       <c r="N5" s="107" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="O5" s="107" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="P5" s="108"/>
       <c r="Q5" s="107" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="R5" s="107" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="S5" s="108"/>
       <c r="T5" s="107" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="U5" s="107" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="V5" s="108"/>
       <c r="W5" s="107" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="X5" s="107" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="Y5" s="107" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="Z5" s="107" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7875,68 +7823,68 @@
       </c>
       <c r="C6" s="108"/>
       <c r="D6" s="111" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="E6" s="111"/>
       <c r="F6" s="111"/>
       <c r="G6" s="108"/>
       <c r="H6" s="110" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="I6" s="108"/>
       <c r="J6" s="110" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="K6" s="108"/>
       <c r="L6" s="110" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="M6" s="15"/>
       <c r="N6" s="110" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="O6" s="110" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="P6" s="108"/>
       <c r="Q6" s="110" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="R6" s="110" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="S6" s="15"/>
       <c r="T6" s="110" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="U6" s="110" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="V6" s="110" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="W6" s="110" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="X6" s="110" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Y6" s="110" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z6" s="110" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="H7" s="112" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="J7" s="112" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="L7" s="112" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7945,7 +7893,7 @@
       </c>
       <c r="C8" s="114"/>
       <c r="D8" s="115" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E8" s="115"/>
       <c r="F8" s="115"/>
@@ -8036,11 +7984,11 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="127" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C10" s="122"/>
       <c r="D10" s="128" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="E10" s="128"/>
       <c r="F10" s="128"/>
@@ -8093,11 +8041,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="127" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C11" s="122"/>
       <c r="D11" s="128" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E11" s="128"/>
       <c r="F11" s="128"/>
@@ -8150,11 +8098,11 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="127" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C12" s="122"/>
       <c r="D12" s="128" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="E12" s="128"/>
       <c r="F12" s="128"/>
@@ -8207,11 +8155,11 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="127" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="C13" s="122"/>
       <c r="D13" s="128" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="E13" s="128"/>
       <c r="F13" s="128"/>
@@ -8264,11 +8212,11 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="127" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C14" s="122"/>
       <c r="D14" s="128" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="E14" s="128"/>
       <c r="F14" s="128"/>
@@ -8427,7 +8375,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="137" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C20" s="138"/>
       <c r="D20" s="138"/>
@@ -8495,7 +8443,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="137" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="C21" s="138"/>
       <c r="D21" s="138"/>
@@ -8563,7 +8511,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="143" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C24" s="66"/>
       <c r="D24" s="66"/>
@@ -8576,16 +8524,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="107" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="C25" s="107" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="D25" s="107" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="E25" s="107" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="F25" s="107" t="s">
         <v>54</v>
@@ -8594,18 +8542,18 @@
         <v>55</v>
       </c>
       <c r="H25" s="107" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="I25" s="107" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="J25" s="107" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="144" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C26" s="145" t="n">
         <f aca="false">U21</f>
@@ -8642,7 +8590,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="149" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="C27" s="150" t="n">
         <f aca="false">X21</f>
@@ -8679,7 +8627,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="144" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C28" s="145" t="n">
         <f aca="false">Z21</f>
@@ -8716,7 +8664,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="154" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -8763,12 +8711,12 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="8" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="8" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8788,7 +8736,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="F8" s="59" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$8*'Sources &amp; Checks'!$B$5</f>
@@ -8797,7 +8745,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="8" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F8/(F8+F15)</f>
@@ -8806,7 +8754,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="F10" s="156" t="n">
         <f aca="false">F11+F14*F13</f>
@@ -8815,7 +8763,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="F11" s="39" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$10</f>
@@ -8824,7 +8772,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="8" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="F12" s="157" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$11</f>
@@ -8833,7 +8781,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="8" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="F13" s="39" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$12</f>
@@ -8842,7 +8790,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="F14" s="158" t="n">
         <f aca="false">1/3*1+2/3*F12</f>
@@ -8854,7 +8802,7 @@
         <v>10</v>
       </c>
       <c r="B15" s="78" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="F15" s="159" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$7</f>
@@ -8863,7 +8811,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="8" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="F16" s="40" t="n">
         <f aca="false">F15/(F15+F8)</f>
@@ -8872,7 +8820,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="8" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="F17" s="40" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$13</f>
@@ -8881,7 +8829,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="F18" s="40" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$14</f>
@@ -8893,7 +8841,7 @@
         <v>10</v>
       </c>
       <c r="B20" s="78" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="F20" s="59" t="n">
         <f aca="false">F15+F8</f>
@@ -8940,7 +8888,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="161" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B1" s="161"/>
       <c r="C1" s="161"/>
@@ -8948,156 +8896,156 @@
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="107" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="B3" s="107" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C3" s="107" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="D3" s="107" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="162" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="B4" s="163" t="n">
         <v>46087</v>
       </c>
       <c r="C4" s="162" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="D4" s="162" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="162" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="B5" s="164" t="n">
         <v>26.19</v>
       </c>
       <c r="C5" s="162" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="D5" s="162" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="162" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B6" s="165" t="n">
         <v>2400</v>
       </c>
       <c r="C6" s="162" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="D6" s="162" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="162" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B7" s="165" t="n">
         <v>1500</v>
       </c>
       <c r="C7" s="162" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="D7" s="162" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="162" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="B8" s="165" t="n">
         <v>1050</v>
       </c>
       <c r="C8" s="162" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="D8" s="162" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="162" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B9" s="165" t="n">
         <v>1066.8</v>
       </c>
       <c r="C9" s="162" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="D9" s="162" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="162" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B10" s="166" t="n">
         <v>0.028643</v>
       </c>
       <c r="C10" s="162" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="D10" s="162" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="162" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="B11" s="167" t="n">
         <v>1.01</v>
       </c>
       <c r="C11" s="162" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="D11" s="162" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="162" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="B12" s="166" t="n">
         <v>0.06</v>
       </c>
       <c r="C12" s="162" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="D12" s="162" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="162" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="B13" s="166" t="n">
         <v>0.03</v>
       </c>
       <c r="C13" s="162" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="D13" s="162" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9108,110 +9056,110 @@
         <v>0.1</v>
       </c>
       <c r="C14" s="162" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="D14" s="162" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="168" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="B16" s="168" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="168" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="B18" s="168" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="C18" s="168" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="D18" s="168" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="168" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="B19" s="169" t="n">
         <v>0.0909</v>
       </c>
       <c r="C19" s="168" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="D19" s="168" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="168" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="B20" s="169" t="n">
         <v>0.1722</v>
       </c>
       <c r="C20" s="168" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="D20" s="168" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="168" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="B21" s="169" t="n">
         <v>0.0805</v>
       </c>
       <c r="C21" s="168" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="D21" s="168" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="168" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="B22" s="169" t="n">
         <v>0.1828</v>
       </c>
       <c r="C22" s="168" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="D22" s="168" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="168" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="B23" s="169" t="n">
         <v>-0.0287</v>
       </c>
       <c r="C23" s="168" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="D23" s="168" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="170" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="B25" s="171" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -9249,21 +9197,21 @@
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="174" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="C3" s="175" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="D3" s="176" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="E3" s="177" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="178" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="C4" s="179" t="n">
         <v>10775</v>
@@ -9277,7 +9225,7 @@
     </row>
     <row r="5" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="182" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="C5" s="183" t="n">
         <v>9332</v>
@@ -9291,7 +9239,7 @@
     </row>
     <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="182" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="C6" s="183" t="n">
         <v>1443</v>
@@ -9305,7 +9253,7 @@
     </row>
     <row r="7" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="186" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="C7" s="187" t="n">
         <v>1314</v>
@@ -9319,21 +9267,21 @@
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="174" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="C10" s="175" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="D10" s="176" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="E10" s="177" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="178" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="C11" s="179" t="n">
         <v>16406</v>
@@ -9347,7 +9295,7 @@
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="182" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="C12" s="183" t="n">
         <v>5643</v>
@@ -9361,7 +9309,7 @@
     </row>
     <row r="13" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="186" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="C13" s="187" t="n">
         <v>4675</v>
@@ -9375,21 +9323,21 @@
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="174" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C16" s="175" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="D16" s="176" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="E16" s="177" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="178" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="C17" s="179" t="n">
         <v>7422</v>
@@ -9403,7 +9351,7 @@
     </row>
     <row r="18" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="182" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="C18" s="183" t="n">
         <v>3341</v>
@@ -9417,7 +9365,7 @@
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="190" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="C19" s="191" t="n">
         <f aca="false">C17+C18</f>
@@ -9434,21 +9382,21 @@
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="174" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="C22" s="175" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="D22" s="176" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="E22" s="177" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="178" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="C23" s="194" t="n">
         <f aca="false">(C4-4800.9)/4800.9</f>
@@ -9465,10 +9413,10 @@
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="182" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="C24" s="196" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="D24" s="197" t="n">
         <f aca="false">(D7-C7)/C7</f>
@@ -9481,7 +9429,7 @@
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="182" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="C25" s="199" t="n">
         <f aca="false">C7/C4</f>
@@ -9498,7 +9446,7 @@
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="182" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="C26" s="199" t="n">
         <f aca="false">(C4-C5)/C4</f>
@@ -9515,7 +9463,7 @@
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="182" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="C27" s="199" t="n">
         <f aca="false">C5/C4</f>
@@ -9532,7 +9480,7 @@
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="182" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="C28" s="199" t="n">
         <f aca="false">C7/C11</f>
@@ -9549,7 +9497,7 @@
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="182" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="C29" s="199" t="n">
         <f aca="false">C7/C12</f>
@@ -9566,7 +9514,7 @@
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="182" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C30" s="199" t="n">
         <f aca="false">C19/C11</f>
@@ -9583,7 +9531,7 @@
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="186" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="C31" s="200" t="n">
         <f aca="false">C12/C11</f>
@@ -9600,17 +9548,17 @@
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="172" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="172" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="172" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -9642,12 +9590,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="84" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="86" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="C3" s="86"/>
     </row>
@@ -9662,7 +9610,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="91" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="C5" s="95" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$21</f>
@@ -9671,7 +9619,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="91" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="C6" s="95" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$22</f>
@@ -9680,7 +9628,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="91" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="C7" s="95" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$23</f>
@@ -9689,7 +9637,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="91" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="C8" s="96" t="n">
         <f aca="false">DCF!$N$20</f>
@@ -9698,7 +9646,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="91" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="C9" s="96" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$6</f>
@@ -9707,7 +9655,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="91" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="C10" s="96" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$7</f>
@@ -9716,7 +9664,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="91" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="C11" s="96" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$9</f>
@@ -9734,7 +9682,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="91" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="C13" s="93" t="n">
         <f aca="false">WACC!$F$11+WACC!$F$12*WACC!$F$13</f>
@@ -9743,7 +9691,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="91" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="C14" s="93" t="n">
         <f aca="false">WACC!$F$9*C13+WACC!$F$16*WACC!$F$17*(1-WACC!$F$18)</f>
@@ -9752,12 +9700,12 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="204" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="86" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="C17" s="86"/>
       <c r="D17" s="86"/>
@@ -9776,13 +9724,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C18" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E18" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F18" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -9830,14 +9778,14 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C19" s="95" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E19" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F19" s="207" t="n">
         <f aca="false">$C$19</f>
@@ -9882,7 +9830,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C20" s="95" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -9941,7 +9889,7 @@
         <v>0.0860234789737754</v>
       </c>
       <c r="E21" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F21" s="208" t="n">
         <f aca="false">F20*$C$20*(1-$C$4)</f>
@@ -9990,7 +9938,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C22" s="95" t="n">
         <f aca="false">DCF!$L$17</f>
@@ -10046,7 +9994,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C23" s="209" t="n">
         <v>0</v>
@@ -10101,13 +10049,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C24" s="209" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F24" s="208" t="n">
         <f aca="false">F21*F23</f>
@@ -10152,7 +10100,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C25" s="209" t="n">
         <v>0</v>
@@ -10214,7 +10162,7 @@
         <v>13045.07390491</v>
       </c>
       <c r="E26" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F26" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -10266,7 +10214,7 @@
         <v>38722.0828951123</v>
       </c>
       <c r="E27" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F27" s="208" t="n">
         <f aca="false">F25/(1+$C$21)^F26</f>
@@ -10329,7 +10277,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C30" s="96" t="n">
         <f aca="false">C29+$C$9-$C$10</f>
@@ -10356,7 +10304,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C33" s="97" t="n">
         <f aca="false">C28/C29</f>
@@ -10365,7 +10313,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="86" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="C36" s="86"/>
       <c r="D36" s="86"/>
@@ -10384,13 +10332,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C37" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E37" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F37" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -10438,14 +10386,14 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C38" s="95" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E38" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F38" s="207" t="n">
         <f aca="false">$C$38</f>
@@ -10490,7 +10438,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C39" s="95" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -10549,7 +10497,7 @@
         <v>0.0858338239797238</v>
       </c>
       <c r="E40" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F40" s="208" t="n">
         <f aca="false">F39*$C$39*(1-$C$4)</f>
@@ -10598,7 +10546,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C41" s="95" t="n">
         <f aca="false">DCF!$L$17</f>
@@ -10654,7 +10602,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C42" s="209" t="n">
         <v>0</v>
@@ -10709,13 +10657,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C43" s="209" t="n">
         <v>0</v>
       </c>
       <c r="E43" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F43" s="208" t="n">
         <f aca="false">F40*F42</f>
@@ -10760,7 +10708,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C44" s="209" t="n">
         <v>0</v>
@@ -10822,7 +10770,7 @@
         <v>13054.5731443257</v>
       </c>
       <c r="E45" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F45" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -10874,7 +10822,7 @@
         <v>38825.7598673345</v>
       </c>
       <c r="E46" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F46" s="208" t="n">
         <f aca="false">F44/(1+$C$40)^F45</f>
@@ -10937,7 +10885,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C49" s="96" t="n">
         <f aca="false">C48+$C$9-$C$10</f>
@@ -10964,7 +10912,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C52" s="97" t="n">
         <f aca="false">C47/C48</f>
@@ -10973,7 +10921,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="86" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="C55" s="86"/>
       <c r="D55" s="86"/>
@@ -10992,13 +10940,13 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C56" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E56" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F56" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -11046,14 +10994,14 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C57" s="95" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E57" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F57" s="207" t="n">
         <f aca="false">$C$57</f>
@@ -11098,7 +11046,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C58" s="95" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -11157,7 +11105,7 @@
         <v>0.0860234789737754</v>
       </c>
       <c r="E59" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F59" s="208" t="n">
         <f aca="false">F58*$C$58*(1-$C$4)</f>
@@ -11206,7 +11154,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B60" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C60" s="95" t="n">
         <f aca="false">DCF!$L$17</f>
@@ -11262,7 +11210,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B61" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C61" s="209" t="n">
         <v>0</v>
@@ -11317,13 +11265,13 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B62" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C62" s="209" t="n">
         <v>1</v>
       </c>
       <c r="E62" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F62" s="208" t="n">
         <f aca="false">F59*F61</f>
@@ -11368,7 +11316,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B63" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C63" s="209" t="n">
         <v>0</v>
@@ -11430,7 +11378,7 @@
         <v>13045.07390491</v>
       </c>
       <c r="E64" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F64" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -11482,7 +11430,7 @@
         <v>60883.781787047</v>
       </c>
       <c r="E65" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F65" s="208" t="n">
         <f aca="false">F63/(1+$C$59)^F64</f>
@@ -11545,7 +11493,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B68" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C68" s="96" t="n">
         <f aca="false">C67+$C$9-$C$10</f>
@@ -11572,7 +11520,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B71" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C71" s="97" t="n">
         <f aca="false">C66/C67</f>
@@ -11581,7 +11529,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B74" s="86" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="C74" s="86"/>
       <c r="D74" s="86"/>
@@ -11600,13 +11548,13 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B75" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C75" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E75" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F75" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -11654,14 +11602,14 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B76" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C76" s="95" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E76" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F76" s="207" t="n">
         <f aca="false">$C$76</f>
@@ -11706,7 +11654,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B77" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C77" s="95" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -11765,7 +11713,7 @@
         <v>0.0858338239797238</v>
       </c>
       <c r="E78" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F78" s="208" t="n">
         <f aca="false">F77*$C$77*(1-$C$4)</f>
@@ -11814,7 +11762,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B79" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C79" s="95" t="n">
         <f aca="false">DCF!$L$17</f>
@@ -11870,7 +11818,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B80" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C80" s="209" t="n">
         <v>0</v>
@@ -11925,13 +11873,13 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B81" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C81" s="209" t="n">
         <v>1</v>
       </c>
       <c r="E81" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F81" s="208" t="n">
         <f aca="false">F78*F80</f>
@@ -11976,7 +11924,7 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B82" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C82" s="209" t="n">
         <v>0</v>
@@ -12038,7 +11986,7 @@
         <v>13054.5731443257</v>
       </c>
       <c r="E83" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F83" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -12090,7 +12038,7 @@
         <v>61018.3081629823</v>
       </c>
       <c r="E84" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F84" s="208" t="n">
         <f aca="false">F82/(1+$C$78)^F83</f>
@@ -12153,7 +12101,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B87" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C87" s="96" t="n">
         <f aca="false">C86+$C$9-$C$10</f>
@@ -12180,7 +12128,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B90" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C90" s="97" t="n">
         <f aca="false">C85/C86</f>
@@ -12189,7 +12137,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B93" s="86" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="C93" s="86"/>
       <c r="D93" s="86"/>
@@ -12208,13 +12156,13 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B94" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C94" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E94" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F94" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -12262,14 +12210,14 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B95" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C95" s="95" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E95" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F95" s="207" t="n">
         <f aca="false">$C$95</f>
@@ -12314,7 +12262,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B96" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C96" s="95" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -12373,7 +12321,7 @@
         <v>0.0858338239797238</v>
       </c>
       <c r="E97" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F97" s="208" t="n">
         <f aca="false">F96*$C$96*(1-$C$4)</f>
@@ -12422,7 +12370,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B98" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C98" s="95" t="n">
         <f aca="false">DCF!$L$17</f>
@@ -12478,7 +12426,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B99" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C99" s="209" t="n">
         <v>1</v>
@@ -12533,13 +12481,13 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B100" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C100" s="209" t="n">
         <v>1</v>
       </c>
       <c r="E100" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F100" s="208" t="n">
         <f aca="false">F97*F99</f>
@@ -12584,7 +12532,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B101" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C101" s="209" t="n">
         <v>0</v>
@@ -12646,7 +12594,7 @@
         <v>11516.4871200723</v>
       </c>
       <c r="E102" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F102" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -12698,7 +12646,7 @@
         <v>42710.8785354486</v>
       </c>
       <c r="E103" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F103" s="208" t="n">
         <f aca="false">F101/(1+$C$97)^F102</f>
@@ -12761,7 +12709,7 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B106" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C106" s="96" t="n">
         <f aca="false">C105+$C$9-$C$10</f>
@@ -12788,7 +12736,7 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B109" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C109" s="97" t="n">
         <f aca="false">C104/C105</f>
@@ -12797,7 +12745,7 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B112" s="86" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="C112" s="86"/>
       <c r="D112" s="86"/>
@@ -12816,13 +12764,13 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B113" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C113" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E113" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F113" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -12870,14 +12818,14 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B114" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C114" s="95" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E114" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F114" s="207" t="n">
         <f aca="false">$C$114</f>
@@ -12922,7 +12870,7 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B115" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C115" s="95" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -12981,7 +12929,7 @@
         <v>0.0858338239797238</v>
       </c>
       <c r="E116" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F116" s="208" t="n">
         <f aca="false">F115*$C$115*(1-$C$4)</f>
@@ -13030,7 +12978,7 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B117" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C117" s="95" t="n">
         <f aca="false">DCF!$L$17</f>
@@ -13086,7 +13034,7 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B118" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C118" s="209" t="n">
         <v>1</v>
@@ -13141,13 +13089,13 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B119" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C119" s="209" t="n">
         <v>1</v>
       </c>
       <c r="E119" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F119" s="208" t="n">
         <f aca="false">F116*F118</f>
@@ -13192,7 +13140,7 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B120" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C120" s="209" t="n">
         <v>1</v>
@@ -13254,7 +13202,7 @@
         <v>13846.0199602466</v>
       </c>
       <c r="E121" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F121" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -13306,7 +13254,7 @@
         <v>42710.8785354486</v>
       </c>
       <c r="E122" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F122" s="208" t="n">
         <f aca="false">F120/(1+$C$116)^F121</f>
@@ -13369,7 +13317,7 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B125" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C125" s="96" t="n">
         <f aca="false">C124+$C$9-$C$10</f>
@@ -13396,7 +13344,7 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B128" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C128" s="97" t="n">
         <f aca="false">C123/C124</f>
@@ -13405,7 +13353,7 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B131" s="204" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13429,13 +13377,13 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B133" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C133" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E133" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F133" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -13483,14 +13431,14 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B134" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C134" s="95" t="n">
         <f aca="false">DCF!$H$11</f>
         <v>0.07</v>
       </c>
       <c r="E134" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F134" s="207" t="n">
         <f aca="false">$C$134</f>
@@ -13535,7 +13483,7 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B135" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C135" s="95" t="n">
         <f aca="false">DCF!$H$13</f>
@@ -13594,7 +13542,7 @@
         <v>0.092</v>
       </c>
       <c r="E136" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F136" s="208" t="n">
         <f aca="false">F135*$C$135*(1-$C$4)</f>
@@ -13643,7 +13591,7 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B137" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C137" s="95" t="n">
         <f aca="false">DCF!$H$17</f>
@@ -13699,7 +13647,7 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B138" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C138" s="209" t="n">
         <v>1</v>
@@ -13754,13 +13702,13 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B139" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C139" s="209" t="n">
         <v>1</v>
       </c>
       <c r="E139" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F139" s="208" t="n">
         <f aca="false">F136*F138</f>
@@ -13805,7 +13753,7 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B140" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C140" s="209" t="n">
         <v>1</v>
@@ -13867,7 +13815,7 @@
         <v>11975.9526815862</v>
       </c>
       <c r="E141" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F141" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -13919,7 +13867,7 @@
         <v>32585.2141029511</v>
       </c>
       <c r="E142" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F142" s="208" t="n">
         <f aca="false">F140/(1+$C$136)^F141</f>
@@ -13982,7 +13930,7 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B145" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C145" s="96" t="n">
         <f aca="false">C144+$C$9-$C$10</f>
@@ -14009,7 +13957,7 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B148" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C148" s="97" t="n">
         <f aca="false">C143/C144</f>
@@ -14037,13 +13985,13 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B152" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C152" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E152" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F152" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -14091,14 +14039,14 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B153" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C153" s="95" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E153" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F153" s="207" t="n">
         <f aca="false">$C$153</f>
@@ -14143,7 +14091,7 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B154" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C154" s="95" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -14202,7 +14150,7 @@
         <v>0.0858338239797238</v>
       </c>
       <c r="E155" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F155" s="208" t="n">
         <f aca="false">F154*$C$154*(1-$C$4)</f>
@@ -14251,7 +14199,7 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B156" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C156" s="95" t="n">
         <f aca="false">DCF!$L$17</f>
@@ -14307,7 +14255,7 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B157" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C157" s="209" t="n">
         <v>1</v>
@@ -14362,13 +14310,13 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B158" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C158" s="209" t="n">
         <v>1</v>
       </c>
       <c r="E158" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F158" s="208" t="n">
         <f aca="false">F155*F157</f>
@@ -14413,7 +14361,7 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B159" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C159" s="209" t="n">
         <v>1</v>
@@ -14475,7 +14423,7 @@
         <v>13846.0199602466</v>
       </c>
       <c r="E160" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F160" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -14527,7 +14475,7 @@
         <v>42710.8785354486</v>
       </c>
       <c r="E161" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F161" s="208" t="n">
         <f aca="false">F159/(1+$C$155)^F160</f>
@@ -14590,7 +14538,7 @@
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B164" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C164" s="96" t="n">
         <f aca="false">C163+$C$9-$C$10</f>
@@ -14617,7 +14565,7 @@
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B167" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C167" s="97" t="n">
         <f aca="false">C162/C163</f>
@@ -14645,13 +14593,13 @@
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B171" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C171" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E171" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F171" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -14699,14 +14647,14 @@
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B172" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C172" s="95" t="n">
         <f aca="false">DCF!$P$11</f>
         <v>0.11</v>
       </c>
       <c r="E172" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F172" s="207" t="n">
         <f aca="false">$C$172</f>
@@ -14751,7 +14699,7 @@
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B173" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C173" s="95" t="n">
         <f aca="false">DCF!$P$13</f>
@@ -14810,7 +14758,7 @@
         <v>0.082</v>
       </c>
       <c r="E174" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F174" s="208" t="n">
         <f aca="false">F173*$C$173*(1-$C$4)</f>
@@ -14859,7 +14807,7 @@
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B175" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C175" s="95" t="n">
         <f aca="false">DCF!$P$17</f>
@@ -14915,7 +14863,7 @@
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B176" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C176" s="209" t="n">
         <v>1</v>
@@ -14970,13 +14918,13 @@
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B177" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C177" s="209" t="n">
         <v>1</v>
       </c>
       <c r="E177" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F177" s="208" t="n">
         <f aca="false">F174*F176</f>
@@ -15021,7 +14969,7 @@
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B178" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C178" s="209" t="n">
         <v>1</v>
@@ -15083,7 +15031,7 @@
         <v>15963.3087683037</v>
       </c>
       <c r="E179" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F179" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -15135,7 +15083,7 @@
         <v>54031.0813221065</v>
       </c>
       <c r="E180" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F180" s="208" t="n">
         <f aca="false">F178/(1+$C$174)^F179</f>
@@ -15198,7 +15146,7 @@
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B183" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C183" s="96" t="n">
         <f aca="false">C182+$C$9-$C$10</f>
@@ -15225,7 +15173,7 @@
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B186" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C186" s="97" t="n">
         <f aca="false">C181/C182</f>
@@ -15234,7 +15182,7 @@
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B189" s="86" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="C189" s="86"/>
       <c r="D189" s="86"/>
@@ -15253,13 +15201,13 @@
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B190" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C190" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E190" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F190" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -15307,14 +15255,14 @@
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B191" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C191" s="95" t="n">
         <f aca="false">DCF!$H$11</f>
         <v>0.07</v>
       </c>
       <c r="E191" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F191" s="207" t="n">
         <f aca="false">$C$191</f>
@@ -15359,7 +15307,7 @@
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B192" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C192" s="95" t="n">
         <f aca="false">DCF!$H$13</f>
@@ -15418,7 +15366,7 @@
         <v>0.092</v>
       </c>
       <c r="E193" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F193" s="208" t="n">
         <f aca="false">F192*$C$192*(1-$C$4)</f>
@@ -15467,7 +15415,7 @@
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B194" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C194" s="95" t="n">
         <f aca="false">DCF!$H$17</f>
@@ -15523,7 +15471,7 @@
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B195" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C195" s="209" t="n">
         <v>0</v>
@@ -15578,13 +15526,13 @@
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B196" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C196" s="209" t="n">
         <v>0</v>
       </c>
       <c r="E196" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F196" s="208" t="n">
         <f aca="false">F193*F195</f>
@@ -15629,7 +15577,7 @@
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B197" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C197" s="209" t="n">
         <v>0</v>
@@ -15691,7 +15639,7 @@
         <v>9931.09819247139</v>
       </c>
       <c r="E198" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F198" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -15743,7 +15691,7 @@
         <v>23792.7950795298</v>
       </c>
       <c r="E199" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F199" s="208" t="n">
         <f aca="false">F197/(1+$C$193)^F198</f>
@@ -15806,7 +15754,7 @@
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B202" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C202" s="96" t="n">
         <f aca="false">C201+$C$9-$C$10</f>
@@ -15833,7 +15781,7 @@
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B205" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C205" s="97" t="n">
         <f aca="false">C200/C201</f>
@@ -15842,7 +15790,7 @@
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B208" s="86" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="C208" s="86"/>
       <c r="D208" s="86"/>
@@ -15861,13 +15809,13 @@
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B209" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C209" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E209" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F209" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -15915,14 +15863,14 @@
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B210" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C210" s="95" t="n">
         <f aca="false">DCF!$P$11</f>
         <v>0.11</v>
       </c>
       <c r="E210" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F210" s="207" t="n">
         <f aca="false">$C$210</f>
@@ -15967,7 +15915,7 @@
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B211" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C211" s="95" t="n">
         <f aca="false">DCF!$P$13</f>
@@ -16026,7 +15974,7 @@
         <v>0.082</v>
       </c>
       <c r="E212" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F212" s="208" t="n">
         <f aca="false">F211*$C$211*(1-$C$4)</f>
@@ -16075,7 +16023,7 @@
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B213" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C213" s="95" t="n">
         <f aca="false">DCF!$P$17</f>
@@ -16131,7 +16079,7 @@
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B214" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C214" s="209" t="n">
         <v>0</v>
@@ -16186,13 +16134,13 @@
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B215" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C215" s="209" t="n">
         <v>0</v>
       </c>
       <c r="E215" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F215" s="208" t="n">
         <f aca="false">F212*F214</f>
@@ -16237,7 +16185,7 @@
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B216" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C216" s="209" t="n">
         <v>0</v>
@@ -16299,7 +16247,7 @@
         <v>16684.3795279921</v>
       </c>
       <c r="E217" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F217" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -16351,7 +16299,7 @@
         <v>60531.5076403291</v>
       </c>
       <c r="E218" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F218" s="208" t="n">
         <f aca="false">F216/(1+$C$212)^F217</f>
@@ -16414,7 +16362,7 @@
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B221" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C221" s="96" t="n">
         <f aca="false">C220+$C$9-$C$10</f>
@@ -16441,7 +16389,7 @@
     </row>
     <row r="224" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B224" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C224" s="97" t="n">
         <f aca="false">C219/C220</f>
@@ -16450,12 +16398,12 @@
     </row>
     <row r="227" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B227" s="204" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B228" s="86" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="C228" s="86"/>
       <c r="D228" s="86"/>
@@ -16474,13 +16422,13 @@
     </row>
     <row r="229" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B229" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C229" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E229" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F229" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -16528,14 +16476,14 @@
     </row>
     <row r="230" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B230" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C230" s="95" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E230" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F230" s="207" t="n">
         <f aca="false">$C$230</f>
@@ -16580,7 +16528,7 @@
     </row>
     <row r="231" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B231" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C231" s="95" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -16639,7 +16587,7 @@
         <v>0.0858338239797238</v>
       </c>
       <c r="E232" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F232" s="208" t="n">
         <f aca="false">F231*$C$231*(1-$C$4)</f>
@@ -16688,7 +16636,7 @@
     </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B233" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C233" s="95" t="n">
         <f aca="false">DCF!$D$92</f>
@@ -16744,7 +16692,7 @@
     </row>
     <row r="234" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B234" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C234" s="209" t="n">
         <v>1</v>
@@ -16799,13 +16747,13 @@
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B235" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C235" s="209" t="n">
         <v>1</v>
       </c>
       <c r="E235" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F235" s="208" t="n">
         <f aca="false">F232*F234</f>
@@ -16850,7 +16798,7 @@
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B236" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C236" s="209" t="n">
         <v>1</v>
@@ -16912,7 +16860,7 @@
         <v>14476.5499935888</v>
       </c>
       <c r="E237" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F237" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -16964,7 +16912,7 @@
         <v>40292.985457408</v>
       </c>
       <c r="E238" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F238" s="208" t="n">
         <f aca="false">F236/(1+$C$232)^F237</f>
@@ -17027,7 +16975,7 @@
     </row>
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B241" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C241" s="96" t="n">
         <f aca="false">C240+$C$9-$C$10</f>
@@ -17054,7 +17002,7 @@
     </row>
     <row r="244" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B244" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C244" s="97" t="n">
         <f aca="false">C239/C240</f>
@@ -17063,7 +17011,7 @@
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B247" s="86" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C247" s="86"/>
       <c r="D247" s="86"/>
@@ -17082,13 +17030,13 @@
     </row>
     <row r="248" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B248" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C248" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E248" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F248" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -17136,14 +17084,14 @@
     </row>
     <row r="249" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B249" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C249" s="95" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E249" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F249" s="207" t="n">
         <f aca="false">$C$249</f>
@@ -17188,7 +17136,7 @@
     </row>
     <row r="250" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B250" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C250" s="95" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -17247,7 +17195,7 @@
         <v>0.0858338239797238</v>
       </c>
       <c r="E251" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F251" s="208" t="n">
         <f aca="false">F250*$C$250*(1-$C$4)</f>
@@ -17296,7 +17244,7 @@
     </row>
     <row r="252" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B252" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C252" s="95" t="n">
         <f aca="false">DCF!$F$92</f>
@@ -17352,7 +17300,7 @@
     </row>
     <row r="253" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B253" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C253" s="209" t="n">
         <v>1</v>
@@ -17407,13 +17355,13 @@
     </row>
     <row r="254" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B254" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C254" s="209" t="n">
         <v>1</v>
       </c>
       <c r="E254" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F254" s="208" t="n">
         <f aca="false">F251*F253</f>
@@ -17458,7 +17406,7 @@
     </row>
     <row r="255" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B255" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C255" s="209" t="n">
         <v>1</v>
@@ -17520,7 +17468,7 @@
         <v>14166.8536766156</v>
       </c>
       <c r="E256" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F256" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -17572,7 +17520,7 @@
         <v>41486.5594951797</v>
       </c>
       <c r="E257" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F257" s="208" t="n">
         <f aca="false">F255/(1+$C$251)^F256</f>
@@ -17635,7 +17583,7 @@
     </row>
     <row r="260" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B260" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C260" s="96" t="n">
         <f aca="false">C259+$C$9-$C$10</f>
@@ -17662,7 +17610,7 @@
     </row>
     <row r="263" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B263" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C263" s="97" t="n">
         <f aca="false">C258/C259</f>
@@ -17671,7 +17619,7 @@
     </row>
     <row r="266" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B266" s="86" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="C266" s="86"/>
       <c r="D266" s="86"/>
@@ -17690,13 +17638,13 @@
     </row>
     <row r="267" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B267" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C267" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E267" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F267" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -17744,14 +17692,14 @@
     </row>
     <row r="268" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B268" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C268" s="95" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E268" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F268" s="207" t="n">
         <f aca="false">$C$268</f>
@@ -17796,7 +17744,7 @@
     </row>
     <row r="269" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B269" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C269" s="95" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -17855,7 +17803,7 @@
         <v>0.0858338239797238</v>
       </c>
       <c r="E270" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F270" s="208" t="n">
         <f aca="false">F269*$C$269*(1-$C$4)</f>
@@ -17904,7 +17852,7 @@
     </row>
     <row r="271" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B271" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C271" s="95" t="n">
         <f aca="false">DCF!$H$92</f>
@@ -17960,7 +17908,7 @@
     </row>
     <row r="272" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B272" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C272" s="209" t="n">
         <v>1</v>
@@ -18015,13 +17963,13 @@
     </row>
     <row r="273" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B273" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C273" s="209" t="n">
         <v>1</v>
       </c>
       <c r="E273" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F273" s="208" t="n">
         <f aca="false">F270*F272</f>
@@ -18066,7 +18014,7 @@
     </row>
     <row r="274" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B274" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C274" s="209" t="n">
         <v>1</v>
@@ -18128,7 +18076,7 @@
         <v>13846.0199602466</v>
       </c>
       <c r="E275" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F275" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -18180,7 +18128,7 @@
         <v>42710.8785354486</v>
       </c>
       <c r="E276" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F276" s="208" t="n">
         <f aca="false">F274/(1+$C$270)^F275</f>
@@ -18243,7 +18191,7 @@
     </row>
     <row r="279" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B279" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C279" s="96" t="n">
         <f aca="false">C278+$C$9-$C$10</f>
@@ -18270,7 +18218,7 @@
     </row>
     <row r="282" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B282" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C282" s="97" t="n">
         <f aca="false">C277/C278</f>
@@ -18279,7 +18227,7 @@
     </row>
     <row r="285" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B285" s="86" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="C285" s="86"/>
       <c r="D285" s="86"/>
@@ -18298,13 +18246,13 @@
     </row>
     <row r="286" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B286" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C286" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E286" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F286" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -18352,14 +18300,14 @@
     </row>
     <row r="287" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B287" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C287" s="95" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E287" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F287" s="207" t="n">
         <f aca="false">$C$287</f>
@@ -18404,7 +18352,7 @@
     </row>
     <row r="288" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B288" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C288" s="95" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -18463,7 +18411,7 @@
         <v>0.0858338239797238</v>
       </c>
       <c r="E289" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F289" s="208" t="n">
         <f aca="false">F288*$C$288*(1-$C$4)</f>
@@ -18512,7 +18460,7 @@
     </row>
     <row r="290" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B290" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C290" s="95" t="n">
         <f aca="false">DCF!$J$92</f>
@@ -18568,7 +18516,7 @@
     </row>
     <row r="291" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B291" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C291" s="209" t="n">
         <v>1</v>
@@ -18623,13 +18571,13 @@
     </row>
     <row r="292" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B292" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C292" s="209" t="n">
         <v>1</v>
       </c>
       <c r="E292" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F292" s="208" t="n">
         <f aca="false">F289*F291</f>
@@ -18674,7 +18622,7 @@
     </row>
     <row r="293" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B293" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C293" s="209" t="n">
         <v>1</v>
@@ -18736,7 +18684,7 @@
         <v>13513.7729723786</v>
       </c>
       <c r="E294" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F294" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -18788,7 +18736,7 @@
         <v>43966.6206249201</v>
       </c>
       <c r="E295" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F295" s="208" t="n">
         <f aca="false">F293/(1+$C$289)^F294</f>
@@ -18851,7 +18799,7 @@
     </row>
     <row r="298" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B298" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C298" s="96" t="n">
         <f aca="false">C297+$C$9-$C$10</f>
@@ -18878,7 +18826,7 @@
     </row>
     <row r="301" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B301" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C301" s="97" t="n">
         <f aca="false">C296/C297</f>
@@ -18887,7 +18835,7 @@
     </row>
     <row r="304" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B304" s="86" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="C304" s="86"/>
       <c r="D304" s="86"/>
@@ -18906,13 +18854,13 @@
     </row>
     <row r="305" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B305" s="205" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C305" s="205" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E305" s="205" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="F305" s="206" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -18960,14 +18908,14 @@
     </row>
     <row r="306" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B306" s="91" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C306" s="95" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E306" s="91" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F306" s="207" t="n">
         <f aca="false">$C$306</f>
@@ -19012,7 +18960,7 @@
     </row>
     <row r="307" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B307" s="91" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C307" s="95" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -19071,7 +19019,7 @@
         <v>0.0858338239797238</v>
       </c>
       <c r="E308" s="91" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="F308" s="208" t="n">
         <f aca="false">F307*$C$307*(1-$C$4)</f>
@@ -19120,7 +19068,7 @@
     </row>
     <row r="309" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B309" s="91" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C309" s="95" t="n">
         <f aca="false">DCF!$L$92</f>
@@ -19176,7 +19124,7 @@
     </row>
     <row r="310" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B310" s="91" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C310" s="209" t="n">
         <v>1</v>
@@ -19231,13 +19179,13 @@
     </row>
     <row r="311" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B311" s="91" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C311" s="209" t="n">
         <v>1</v>
       </c>
       <c r="E311" s="91" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F311" s="208" t="n">
         <f aca="false">F308*F310</f>
@@ -19282,7 +19230,7 @@
     </row>
     <row r="312" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B312" s="91" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C312" s="209" t="n">
         <v>1</v>
@@ -19344,7 +19292,7 @@
         <v>13169.8313946416</v>
       </c>
       <c r="E313" s="91" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="F313" s="212" t="n">
         <f aca="false">DCF!O$71</f>
@@ -19396,7 +19344,7 @@
         <v>45254.4763666792</v>
       </c>
       <c r="E314" s="91" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="F314" s="208" t="n">
         <f aca="false">F312/(1+$C$308)^F313</f>
@@ -19459,7 +19407,7 @@
     </row>
     <row r="317" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B317" s="91" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C317" s="96" t="n">
         <f aca="false">C316+$C$9-$C$10</f>
@@ -19486,7 +19434,7 @@
     </row>
     <row r="320" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B320" s="91" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C320" s="97" t="n">
         <f aca="false">C315/C316</f>

</xml_diff>

<commit_message>
Correct debt to include leases already
</commit_message>
<xml_diff>
--- a/Ryanair_DCF_Model_Kodickova_2026.xlsx
+++ b/Ryanair_DCF_Model_Kodickova_2026.xlsx
@@ -203,7 +203,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Gross debt (1,500) plus lease liabilities (111.2) at 31 Dec 2025, linked to the Sources &amp; Checks sheet.</t>
+          <t xml:space="preserve">Gross debt of 1,500 at 31 Dec 2025, which includes lease liabilities, linked to the Sources &amp; Checks sheet.</t>
         </r>
       </text>
     </comment>
@@ -285,9 +285,10 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
     <author>Unknown Author</author>
+    <author>Viktorie Kodickova</author>
   </authors>
   <commentList>
-    <comment ref="F8" authorId="0">
+    <comment ref="F8" authorId="1">
       <text>
         <r>
           <rPr>
@@ -459,7 +460,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="259">
   <si>
     <t xml:space="preserve">DCF Model - Ryanair</t>
   </si>
@@ -626,7 +627,7 @@
     <t xml:space="preserve">(+) Cash</t>
   </si>
   <si>
-    <t xml:space="preserve">(-) Debt and leases</t>
+    <t xml:space="preserve">(-) Debt (incl. leases)</t>
   </si>
   <si>
     <t xml:space="preserve">Equity Value</t>
@@ -725,15 +726,6 @@
     <t xml:space="preserve">Only the 25 days between the valuation date and the FY26 year end are counted.</t>
   </si>
   <si>
-    <t xml:space="preserve">Equity bridge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sources &amp; Checks!B24, DCF!S77</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lease liabilities of 111.2 (Q3 FY26 balance sheet) are deducted together with gross debt.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Comps</t>
   </si>
   <si>
@@ -881,7 +873,7 @@
     <t xml:space="preserve">EV/EBIT (FY25)</t>
   </si>
   <si>
-    <t xml:space="preserve">Note: Peer medians exclude Ryanair (EX-RYA). Implied EV = Multiple × Ryanair metric. Net Debt Bridge: (+) Cash €2,400M, (−) Debt €1,500M and leases €111M. Shares: 1,066.8M diluted. Large discount vs DCF reflects Ryanair's structurally superior margins vs legacy carriers — direct comps multiples understate intrinsic value.</t>
+    <t xml:space="preserve">Note: Peer medians exclude Ryanair (EX-RYA). Implied EV = Multiple × Ryanair metric. Net Debt Bridge: (+) Cash €2,400M, (−) Debt €1,500M. Shares: 1,066.8M diluted. Large discount vs DCF reflects Ryanair's structurally superior margins vs legacy carriers — direct comps multiples understate intrinsic value.</t>
   </si>
   <si>
     <t xml:space="preserve">WACC = % of equity x cost of equity + % of debt x cost of debt x (1- Tax Rate)</t>
@@ -965,7 +957,7 @@
     <t xml:space="preserve">Gross debt</t>
   </si>
   <si>
-    <t xml:space="preserve">Ryanair Q3 FY26 results: gross debt at 31 Dec 2025.</t>
+    <t xml:space="preserve">Q3 FY26 results: gross debt of €1.5bn at 31 Dec 2025, which includes lease liabilities (balance sheet: debt 1,346.4 + leases 111.2 = 1,457.6).</t>
   </si>
   <si>
     <t xml:space="preserve">Basic shares outstanding</t>
@@ -1058,12 +1050,6 @@
     <t xml:space="preserve">Avg of FY17-FY19 + FY24-FY25 change in net working capital as % of Revenue (negative = cash source, typical for airlines)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lease liabilities</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q3 FY26 results balance sheet at 31 Dec 2025: current 35.3 + non-current 75.9. Added to gross debt in the equity bridge.</t>
-  </si>
-  <si>
     <t xml:space="preserve">⚠ Data Note</t>
   </si>
   <si>
@@ -1178,7 +1164,7 @@
     <t xml:space="preserve">Cash (EUR m)</t>
   </si>
   <si>
-    <t xml:space="preserve">Debt and leases (EUR m)</t>
+    <t xml:space="preserve">Debt incl. leases (EUR m)</t>
   </si>
   <si>
     <t xml:space="preserve">Diluted shares (m)</t>
@@ -1223,7 +1209,7 @@
     <t xml:space="preserve">Enterprise value</t>
   </si>
   <si>
-    <t xml:space="preserve">Equity value (EV + cash - debt and leases)</t>
+    <t xml:space="preserve">Equity value (EV + cash - debt)</t>
   </si>
   <si>
     <t xml:space="preserve">Implied price per share (EUR)</t>
@@ -3171,7 +3157,7 @@
       </c>
       <c r="I5" s="9" t="n">
         <f aca="false">S81</f>
-        <v>31.6198010060632</v>
+        <v>31.7240379764419</v>
       </c>
       <c r="K5" s="8" t="s">
         <v>4</v>
@@ -3210,7 +3196,7 @@
       </c>
       <c r="I7" s="12" t="n">
         <f aca="false">I5/I6-1</f>
-        <v>0.207323444294127</v>
+        <v>0.211303473709121</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6515,8 +6501,8 @@
         <v>55</v>
       </c>
       <c r="S77" s="25" t="n">
-        <f aca="false">'Sources &amp; Checks'!$B$7+'Sources &amp; Checks'!$B$24</f>
-        <v>1611.2</v>
+        <f aca="false">'Sources &amp; Checks'!$B$7</f>
+        <v>1500</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6528,7 +6514,7 @@
       </c>
       <c r="S78" s="25" t="n">
         <f aca="false">S75+S76-S77</f>
-        <v>33732.0037132682</v>
+        <v>33843.2037132682</v>
       </c>
       <c r="T78" s="52"/>
       <c r="U78" s="52"/>
@@ -6554,7 +6540,7 @@
       </c>
       <c r="S81" s="57" t="n">
         <f aca="false">S78/S80</f>
-        <v>31.6198010060632</v>
+        <v>31.7240379764419</v>
       </c>
       <c r="T81" s="58"/>
       <c r="U81" s="58"/>
@@ -6625,11 +6611,11 @@
       </c>
       <c r="L87" s="67" t="n">
         <f aca="false">Calc!$C$29</f>
-        <v>24.7965963086233</v>
+        <v>24.900833279002</v>
       </c>
       <c r="N87" s="65" t="n">
         <f aca="false">L87/'Sources &amp; Checks'!$B$5-1</f>
-        <v>-0.0532036537371797</v>
+        <v>-0.0492236243221853</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6654,11 +6640,11 @@
       </c>
       <c r="L88" s="72" t="n">
         <f aca="false">Calc!$C$48</f>
-        <v>31.6198010060632</v>
+        <v>31.7240379764419</v>
       </c>
       <c r="N88" s="70" t="n">
         <f aca="false">L88/'Sources &amp; Checks'!$B$5-1</f>
-        <v>0.207323444294127</v>
+        <v>0.211303473709121</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6683,11 +6669,11 @@
       </c>
       <c r="L89" s="67" t="n">
         <f aca="false">Calc!$C$67</f>
-        <v>39.2291143805989</v>
+        <v>39.3333513509776</v>
       </c>
       <c r="N89" s="65" t="n">
         <f aca="false">L89/'Sources &amp; Checks'!$B$5-1</f>
-        <v>0.497866146643714</v>
+        <v>0.501846176058708</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6743,24 +6729,24 @@
         <v>0.075</v>
       </c>
       <c r="D93" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$81:$O$81/(1+$B93)^$O$71:$X$71)-(1-$O$70)*Calc!$F$81/(1+$B93)^$O$71+(Calc!$O$77*(1+D$92)*(1-D$92/$B93)/($B93-D$92))/(1+$B93)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>36.1945918474672</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$81:$O$81/(1+$B93)^$O$71:$X$71)-(1-$O$70)*Calc!$F$81/(1+$B93)^$O$71+(Calc!$O$77*(1+D$92)*(1-D$92/$B93)/($B93-D$92))/(1+$B93)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>36.2988288178459</v>
       </c>
       <c r="F93" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$100:$O$100/(1+$B93)^$O$71:$X$71)-(1-$O$70)*Calc!$F$100/(1+$B93)^$O$71+(Calc!$O$96*(1+F$92)*(1-F$92/$B93)/($B93-F$92))/(1+$B93)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>36.5627735935774</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$100:$O$100/(1+$B93)^$O$71:$X$71)-(1-$O$70)*Calc!$F$100/(1+$B93)^$O$71+(Calc!$O$96*(1+F$92)*(1-F$92/$B93)/($B93-F$92))/(1+$B93)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>36.6670105639561</v>
       </c>
       <c r="H93" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$119:$O$119/(1+$B93)^$O$71:$X$71)-(1-$O$70)*Calc!$F$119/(1+$B93)^$O$71+(Calc!$O$115*(1+H$92)*(1-H$92/$B93)/($B93-H$92))/(1+$B93)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>36.9372630299162</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$119:$O$119/(1+$B93)^$O$71:$X$71)-(1-$O$70)*Calc!$F$119/(1+$B93)^$O$71+(Calc!$O$115*(1+H$92)*(1-H$92/$B93)/($B93-H$92))/(1+$B93)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>37.0415000002949</v>
       </c>
       <c r="J93" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$138:$O$138/(1+$B93)^$O$71:$X$71)-(1-$O$70)*Calc!$F$138/(1+$B93)^$O$71+(Calc!$O$134*(1+J$92)*(1-J$92/$B93)/($B93-J$92))/(1+$B93)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>37.3181684611653</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$138:$O$138/(1+$B93)^$O$71:$X$71)-(1-$O$70)*Calc!$F$138/(1+$B93)^$O$71+(Calc!$O$134*(1+J$92)*(1-J$92/$B93)/($B93-J$92))/(1+$B93)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>37.422405431544</v>
       </c>
       <c r="L93" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$157:$O$157/(1+$B93)^$O$71:$X$71)-(1-$O$70)*Calc!$F$157/(1+$B93)^$O$71+(Calc!$O$153*(1+L$92)*(1-L$92/$B93)/($B93-L$92))/(1+$B93)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>37.7055998530035</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$157:$O$157/(1+$B93)^$O$71:$X$71)-(1-$O$70)*Calc!$F$157/(1+$B93)^$O$71+(Calc!$O$153*(1+L$92)*(1-L$92/$B93)/($B93-L$92))/(1+$B93)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>37.8098368233822</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6768,24 +6754,24 @@
         <v>0.08</v>
       </c>
       <c r="D94" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$81:$O$81/(1+$B94)^$O$71:$X$71)-(1-$O$70)*Calc!$F$81/(1+$B94)^$O$71+(Calc!$O$77*(1+D$92)*(1-D$92/$B94)/($B94-D$92))/(1+$B94)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>33.6647173200633</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$81:$O$81/(1+$B94)^$O$71:$X$71)-(1-$O$70)*Calc!$F$81/(1+$B94)^$O$71+(Calc!$O$77*(1+D$92)*(1-D$92/$B94)/($B94-D$92))/(1+$B94)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>33.768954290442</v>
       </c>
       <c r="F94" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$100:$O$100/(1+$B94)^$O$71:$X$71)-(1-$O$70)*Calc!$F$100/(1+$B94)^$O$71+(Calc!$O$96*(1+F$92)*(1-F$92/$B94)/($B94-F$92))/(1+$B94)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>33.9744522914576</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$100:$O$100/(1+$B94)^$O$71:$X$71)-(1-$O$70)*Calc!$F$100/(1+$B94)^$O$71+(Calc!$O$96*(1+F$92)*(1-F$92/$B94)/($B94-F$92))/(1+$B94)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>34.0786892618363</v>
       </c>
       <c r="H94" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$119:$O$119/(1+$B94)^$O$71:$X$71)-(1-$O$70)*Calc!$F$119/(1+$B94)^$O$71+(Calc!$O$115*(1+H$92)*(1-H$92/$B94)/($B94-H$92))/(1+$B94)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>34.289138164529</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$119:$O$119/(1+$B94)^$O$71:$X$71)-(1-$O$70)*Calc!$F$119/(1+$B94)^$O$71+(Calc!$O$115*(1+H$92)*(1-H$92/$B94)/($B94-H$92))/(1+$B94)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>34.3933751349077</v>
       </c>
       <c r="J94" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$138:$O$138/(1+$B94)^$O$71:$X$71)-(1-$O$70)*Calc!$F$138/(1+$B94)^$O$71+(Calc!$O$134*(1+J$92)*(1-J$92/$B94)/($B94-J$92))/(1+$B94)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>34.608855007657</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$138:$O$138/(1+$B94)^$O$71:$X$71)-(1-$O$70)*Calc!$F$138/(1+$B94)^$O$71+(Calc!$O$134*(1+J$92)*(1-J$92/$B94)/($B94-J$92))/(1+$B94)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>34.7130919780357</v>
       </c>
       <c r="L94" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$157:$O$157/(1+$B94)^$O$71:$X$71)-(1-$O$70)*Calc!$F$157/(1+$B94)^$O$71+(Calc!$O$153*(1+L$92)*(1-L$92/$B94)/($B94-L$92))/(1+$B94)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>34.9336840467851</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$157:$O$157/(1+$B94)^$O$71:$X$71)-(1-$O$70)*Calc!$F$157/(1+$B94)^$O$71+(Calc!$O$153*(1+L$92)*(1-L$92/$B94)/($B94-L$92))/(1+$B94)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>35.0379210171638</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6793,24 +6779,24 @@
         <v>0.085</v>
       </c>
       <c r="D95" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$81:$O$81/(1+$B95)^$O$71:$X$71)-(1-$O$70)*Calc!$F$81/(1+$B95)^$O$71+(Calc!$O$77*(1+D$92)*(1-D$92/$B95)/($B95-D$92))/(1+$B95)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>31.4427878941897</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$81:$O$81/(1+$B95)^$O$71:$X$71)-(1-$O$70)*Calc!$F$81/(1+$B95)^$O$71+(Calc!$O$77*(1+D$92)*(1-D$92/$B95)/($B95-D$92))/(1+$B95)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>31.5470248645684</v>
       </c>
       <c r="F95" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$100:$O$100/(1+$B95)^$O$71:$X$71)-(1-$O$70)*Calc!$F$100/(1+$B95)^$O$71+(Calc!$O$96*(1+F$92)*(1-F$92/$B95)/($B95-F$92))/(1+$B95)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>31.7026393213261</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$100:$O$100/(1+$B95)^$O$71:$X$71)-(1-$O$70)*Calc!$F$100/(1+$B95)^$O$71+(Calc!$O$96*(1+F$92)*(1-F$92/$B95)/($B95-F$92))/(1+$B95)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>31.8068762917048</v>
       </c>
       <c r="H95" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$119:$O$119/(1+$B95)^$O$71:$X$71)-(1-$O$70)*Calc!$F$119/(1+$B95)^$O$71+(Calc!$O$115*(1+H$92)*(1-H$92/$B95)/($B95-H$92))/(1+$B95)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>31.9662989725854</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$119:$O$119/(1+$B95)^$O$71:$X$71)-(1-$O$70)*Calc!$F$119/(1+$B95)^$O$71+(Calc!$O$115*(1+H$92)*(1-H$92/$B95)/($B95-H$92))/(1+$B95)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>32.0705359429641</v>
       </c>
       <c r="J95" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$138:$O$138/(1+$B95)^$O$71:$X$71)-(1-$O$70)*Calc!$F$138/(1+$B95)^$O$71+(Calc!$O$134*(1+J$92)*(1-J$92/$B95)/($B95-J$92))/(1+$B95)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>32.2338233203974</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$138:$O$138/(1+$B95)^$O$71:$X$71)-(1-$O$70)*Calc!$F$138/(1+$B95)^$O$71+(Calc!$O$134*(1+J$92)*(1-J$92/$B95)/($B95-J$92))/(1+$B95)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>32.3380602907761</v>
       </c>
       <c r="L95" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$157:$O$157/(1+$B95)^$O$71:$X$71)-(1-$O$70)*Calc!$F$157/(1+$B95)^$O$71+(Calc!$O$153*(1+L$92)*(1-L$92/$B95)/($B95-L$92))/(1+$B95)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>32.5052695762665</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$157:$O$157/(1+$B95)^$O$71:$X$71)-(1-$O$70)*Calc!$F$157/(1+$B95)^$O$71+(Calc!$O$153*(1+L$92)*(1-L$92/$B95)/($B95-L$92))/(1+$B95)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>32.6095065466452</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6819,24 +6805,24 @@
         <v>0.0858027889618787</v>
       </c>
       <c r="D96" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$81:$O$81/(1+$B96)^$O$71:$X$71)-(1-$O$70)*Calc!$F$81/(1+$B96)^$O$71+(Calc!$O$77*(1+D$92)*(1-D$92/$B96)/($B96-D$92))/(1+$B96)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>31.1110914312575</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$81:$O$81/(1+$B96)^$O$71:$X$71)-(1-$O$70)*Calc!$F$81/(1+$B96)^$O$71+(Calc!$O$77*(1+D$92)*(1-D$92/$B96)/($B96-D$92))/(1+$B96)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>31.2153284016362</v>
       </c>
       <c r="F96" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$100:$O$100/(1+$B96)^$O$71:$X$71)-(1-$O$70)*Calc!$F$100/(1+$B96)^$O$71+(Calc!$O$96*(1+F$92)*(1-F$92/$B96)/($B96-F$92))/(1+$B96)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>31.363625223711</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$100:$O$100/(1+$B96)^$O$71:$X$71)-(1-$O$70)*Calc!$F$100/(1+$B96)^$O$71+(Calc!$O$96*(1+F$92)*(1-F$92/$B96)/($B96-F$92))/(1+$B96)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>31.4678621940897</v>
       </c>
       <c r="H96" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$119:$O$119/(1+$B96)^$O$71:$X$71)-(1-$O$70)*Calc!$F$119/(1+$B96)^$O$71+(Calc!$O$115*(1+H$92)*(1-H$92/$B96)/($B96-H$92))/(1+$B96)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>31.6198010060632</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$119:$O$119/(1+$B96)^$O$71:$X$71)-(1-$O$70)*Calc!$F$119/(1+$B96)^$O$71+(Calc!$O$115*(1+H$92)*(1-H$92/$B96)/($B96-H$92))/(1+$B96)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>31.7240379764419</v>
       </c>
       <c r="J96" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$138:$O$138/(1+$B96)^$O$71:$X$71)-(1-$O$70)*Calc!$F$138/(1+$B96)^$O$71+(Calc!$O$134*(1+J$92)*(1-J$92/$B96)/($B96-J$92))/(1+$B96)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>31.8796718349254</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$138:$O$138/(1+$B96)^$O$71:$X$71)-(1-$O$70)*Calc!$F$138/(1+$B96)^$O$71+(Calc!$O$134*(1+J$92)*(1-J$92/$B96)/($B96-J$92))/(1+$B96)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>31.9839088053041</v>
       </c>
       <c r="L96" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$157:$O$157/(1+$B96)^$O$71:$X$71)-(1-$O$70)*Calc!$F$157/(1+$B96)^$O$71+(Calc!$O$153*(1+L$92)*(1-L$92/$B96)/($B96-L$92))/(1+$B96)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>32.1432914456048</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$157:$O$157/(1+$B96)^$O$71:$X$71)-(1-$O$70)*Calc!$F$157/(1+$B96)^$O$71+(Calc!$O$153*(1+L$92)*(1-L$92/$B96)/($B96-L$92))/(1+$B96)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>32.2475284159835</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6844,24 +6830,24 @@
         <v>0.09</v>
       </c>
       <c r="D97" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$81:$O$81/(1+$B97)^$O$71:$X$71)-(1-$O$70)*Calc!$F$81/(1+$B97)^$O$71+(Calc!$O$77*(1+D$92)*(1-D$92/$B97)/($B97-D$92))/(1+$B97)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>29.4771012647604</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$81:$O$81/(1+$B97)^$O$71:$X$71)-(1-$O$70)*Calc!$F$81/(1+$B97)^$O$71+(Calc!$O$77*(1+D$92)*(1-D$92/$B97)/($B97-D$92))/(1+$B97)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>29.5813382351391</v>
       </c>
       <c r="F97" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$100:$O$100/(1+$B97)^$O$71:$X$71)-(1-$O$70)*Calc!$F$100/(1+$B97)^$O$71+(Calc!$O$96*(1+F$92)*(1-F$92/$B97)/($B97-F$92))/(1+$B97)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>29.6941234750103</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$100:$O$100/(1+$B97)^$O$71:$X$71)-(1-$O$70)*Calc!$F$100/(1+$B97)^$O$71+(Calc!$O$96*(1+F$92)*(1-F$92/$B97)/($B97-F$92))/(1+$B97)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>29.798360445389</v>
       </c>
       <c r="H97" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$119:$O$119/(1+$B97)^$O$71:$X$71)-(1-$O$70)*Calc!$F$119/(1+$B97)^$O$71+(Calc!$O$115*(1+H$92)*(1-H$92/$B97)/($B97-H$92))/(1+$B97)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>29.9139867768195</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$119:$O$119/(1+$B97)^$O$71:$X$71)-(1-$O$70)*Calc!$F$119/(1+$B97)^$O$71+(Calc!$O$115*(1+H$92)*(1-H$92/$B97)/($B97-H$92))/(1+$B97)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>30.0182237471982</v>
       </c>
       <c r="J97" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$138:$O$138/(1+$B97)^$O$71:$X$71)-(1-$O$70)*Calc!$F$138/(1+$B97)^$O$71+(Calc!$O$134*(1+J$92)*(1-J$92/$B97)/($B97-J$92))/(1+$B97)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>30.1367278405758</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$138:$O$138/(1+$B97)^$O$71:$X$71)-(1-$O$70)*Calc!$F$138/(1+$B97)^$O$71+(Calc!$O$134*(1+J$92)*(1-J$92/$B97)/($B97-J$92))/(1+$B97)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>30.2409648109546</v>
       </c>
       <c r="L97" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$157:$O$157/(1+$B97)^$O$71:$X$71)-(1-$O$70)*Calc!$F$157/(1+$B97)^$O$71+(Calc!$O$153*(1+L$92)*(1-L$92/$B97)/($B97-L$92))/(1+$B97)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>30.3623837265723</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$157:$O$157/(1+$B97)^$O$71:$X$71)-(1-$O$70)*Calc!$F$157/(1+$B97)^$O$71+(Calc!$O$153*(1+L$92)*(1-L$92/$B97)/($B97-L$92))/(1+$B97)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>30.466620696951</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6869,24 +6855,24 @@
         <v>0.095</v>
       </c>
       <c r="D98" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$81:$O$81/(1+$B98)^$O$71:$X$71)-(1-$O$70)*Calc!$F$81/(1+$B98)^$O$71+(Calc!$O$77*(1+D$92)*(1-D$92/$B98)/($B98-D$92))/(1+$B98)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>27.7268557842724</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$81:$O$81/(1+$B98)^$O$71:$X$71)-(1-$O$70)*Calc!$F$81/(1+$B98)^$O$71+(Calc!$O$77*(1+D$92)*(1-D$92/$B98)/($B98-D$92))/(1+$B98)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>27.8310927546511</v>
       </c>
       <c r="F98" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$100:$O$100/(1+$B98)^$O$71:$X$71)-(1-$O$70)*Calc!$F$100/(1+$B98)^$O$71+(Calc!$O$96*(1+F$92)*(1-F$92/$B98)/($B98-F$92))/(1+$B98)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>27.9069160597402</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$100:$O$100/(1+$B98)^$O$71:$X$71)-(1-$O$70)*Calc!$F$100/(1+$B98)^$O$71+(Calc!$O$96*(1+F$92)*(1-F$92/$B98)/($B98-F$92))/(1+$B98)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>28.0111530301189</v>
       </c>
       <c r="H98" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$119:$O$119/(1+$B98)^$O$71:$X$71)-(1-$O$70)*Calc!$F$119/(1+$B98)^$O$71+(Calc!$O$115*(1+H$92)*(1-H$92/$B98)/($B98-H$92))/(1+$B98)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>28.0889955485976</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$119:$O$119/(1+$B98)^$O$71:$X$71)-(1-$O$70)*Calc!$F$119/(1+$B98)^$O$71+(Calc!$O$115*(1+H$92)*(1-H$92/$B98)/($B98-H$92))/(1+$B98)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>28.1932325189763</v>
       </c>
       <c r="J98" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$138:$O$138/(1+$B98)^$O$71:$X$71)-(1-$O$70)*Calc!$F$138/(1+$B98)^$O$71+(Calc!$O$134*(1+J$92)*(1-J$92/$B98)/($B98-J$92))/(1+$B98)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>28.2731142489404</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$138:$O$138/(1+$B98)^$O$71:$X$71)-(1-$O$70)*Calc!$F$138/(1+$B98)^$O$71+(Calc!$O$134*(1+J$92)*(1-J$92/$B98)/($B98-J$92))/(1+$B98)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>28.3773512193191</v>
       </c>
       <c r="L98" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$157:$O$157/(1+$B98)^$O$71:$X$71)-(1-$O$70)*Calc!$F$157/(1+$B98)^$O$71+(Calc!$O$153*(1+L$92)*(1-L$92/$B98)/($B98-L$92))/(1+$B98)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>28.4592922566704</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$157:$O$157/(1+$B98)^$O$71:$X$71)-(1-$O$70)*Calc!$F$157/(1+$B98)^$O$71+(Calc!$O$153*(1+L$92)*(1-L$92/$B98)/($B98-L$92))/(1+$B98)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>28.5635292270491</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6894,24 +6880,24 @@
         <v>0.1</v>
       </c>
       <c r="D99" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$81:$O$81/(1+$B99)^$O$71:$X$71)-(1-$O$70)*Calc!$F$81/(1+$B99)^$O$71+(Calc!$O$77*(1+D$92)*(1-D$92/$B99)/($B99-D$92))/(1+$B99)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>26.1594245421226</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$81:$O$81/(1+$B99)^$O$71:$X$71)-(1-$O$70)*Calc!$F$81/(1+$B99)^$O$71+(Calc!$O$77*(1+D$92)*(1-D$92/$B99)/($B99-D$92))/(1+$B99)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>26.2636615125014</v>
       </c>
       <c r="F99" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$100:$O$100/(1+$B99)^$O$71:$X$71)-(1-$O$70)*Calc!$F$100/(1+$B99)^$O$71+(Calc!$O$96*(1+F$92)*(1-F$92/$B99)/($B99-F$92))/(1+$B99)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>26.3074442829021</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$100:$O$100/(1+$B99)^$O$71:$X$71)-(1-$O$70)*Calc!$F$100/(1+$B99)^$O$71+(Calc!$O$96*(1+F$92)*(1-F$92/$B99)/($B99-F$92))/(1+$B99)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>26.4116812532808</v>
       </c>
       <c r="H99" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$119:$O$119/(1+$B99)^$O$71:$X$71)-(1-$O$70)*Calc!$F$119/(1+$B99)^$O$71+(Calc!$O$115*(1+H$92)*(1-H$92/$B99)/($B99-H$92))/(1+$B99)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>26.4567825203499</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$119:$O$119/(1+$B99)^$O$71:$X$71)-(1-$O$70)*Calc!$F$119/(1+$B99)^$O$71+(Calc!$O$115*(1+H$92)*(1-H$92/$B99)/($B99-H$92))/(1+$B99)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>26.5610194907286</v>
       </c>
       <c r="J99" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$138:$O$138/(1+$B99)^$O$71:$X$71)-(1-$O$70)*Calc!$F$138/(1+$B99)^$O$71+(Calc!$O$134*(1+J$92)*(1-J$92/$B99)/($B99-J$92))/(1+$B99)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>26.6074451823407</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$138:$O$138/(1+$B99)^$O$71:$X$71)-(1-$O$70)*Calc!$F$138/(1+$B99)^$O$71+(Calc!$O$134*(1+J$92)*(1-J$92/$B99)/($B99-J$92))/(1+$B99)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>26.7116821527194</v>
       </c>
       <c r="L99" s="77" t="n">
-        <f aca="false">(SUMPRODUCT(Calc!$F$157:$O$157/(1+$B99)^$O$71:$X$71)-(1-$O$70)*Calc!$F$157/(1+$B99)^$O$71+(Calc!$O$153*(1+L$92)*(1-L$92/$B99)/($B99-L$92))/(1+$B99)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7-'Sources &amp; Checks'!$B$24)/'Sources &amp; Checks'!$B$9</f>
-        <v>26.759438049799</v>
+        <f aca="false">(SUMPRODUCT(Calc!$F$157:$O$157/(1+$B99)^$O$71:$X$71)-(1-$O$70)*Calc!$F$157/(1+$B99)^$O$71+(Calc!$O$153*(1+L$92)*(1-L$92/$B99)/($B99-L$92))/(1+$B99)^$X$71+'Sources &amp; Checks'!$B$6-'Sources &amp; Checks'!$B$7)/'Sources &amp; Checks'!$B$9</f>
+        <v>26.8636750201777</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6937,7 +6923,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:D10"/>
+  <dimension ref="B1:D9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
@@ -7021,17 +7007,6 @@
       </c>
       <c r="D9" s="83" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="82" t="s">
-        <v>88</v>
-      </c>
-      <c r="C10" s="83" t="s">
-        <v>89</v>
-      </c>
-      <c r="D10" s="83" t="s">
-        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -7067,7 +7042,7 @@
   <sheetData>
     <row r="2" s="2" customFormat="true" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="84" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7084,7 +7059,7 @@
       <c r="L4" s="15"/>
       <c r="M4" s="15"/>
       <c r="N4" s="85" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="O4" s="85"/>
       <c r="P4" s="85"/>
@@ -7092,14 +7067,14 @@
       <c r="R4" s="85"/>
       <c r="S4" s="15"/>
       <c r="T4" s="85" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="U4" s="85"/>
       <c r="V4" s="85"/>
       <c r="W4" s="85"/>
       <c r="X4" s="85"/>
       <c r="Y4" s="86" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="Z4" s="86"/>
     </row>
@@ -7111,49 +7086,49 @@
       <c r="F5" s="33"/>
       <c r="G5" s="33"/>
       <c r="H5" s="87" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I5" s="88"/>
       <c r="J5" s="87" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="K5" s="88"/>
       <c r="L5" s="87" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="M5" s="89"/>
       <c r="N5" s="87" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="O5" s="87" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="P5" s="88"/>
       <c r="Q5" s="87" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="R5" s="87" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="S5" s="88"/>
       <c r="T5" s="87" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="U5" s="87" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="V5" s="88"/>
       <c r="W5" s="87" t="s">
+        <v>101</v>
+      </c>
+      <c r="X5" s="87" t="s">
+        <v>102</v>
+      </c>
+      <c r="Y5" s="87" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z5" s="87" t="s">
         <v>104</v>
-      </c>
-      <c r="X5" s="87" t="s">
-        <v>105</v>
-      </c>
-      <c r="Y5" s="87" t="s">
-        <v>106</v>
-      </c>
-      <c r="Z5" s="87" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7162,68 +7137,68 @@
       </c>
       <c r="C6" s="88"/>
       <c r="D6" s="91" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E6" s="91"/>
       <c r="F6" s="91"/>
       <c r="G6" s="88"/>
       <c r="H6" s="90" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I6" s="88"/>
       <c r="J6" s="90" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="K6" s="88"/>
       <c r="L6" s="90" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="M6" s="15"/>
       <c r="N6" s="90" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="O6" s="90" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="P6" s="88"/>
       <c r="Q6" s="90" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="R6" s="90" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="S6" s="15"/>
       <c r="T6" s="90" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="U6" s="90" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="V6" s="90" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="W6" s="90" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="X6" s="90" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="Y6" s="90" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="Z6" s="90" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="H7" s="92" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="J7" s="92" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="L7" s="92" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7232,7 +7207,7 @@
       </c>
       <c r="C8" s="94"/>
       <c r="D8" s="95" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E8" s="95"/>
       <c r="F8" s="95"/>
@@ -7248,8 +7223,8 @@
       </c>
       <c r="K8" s="94"/>
       <c r="L8" s="97" t="n">
-        <f aca="false">J8-'Sources &amp; Checks'!$B$6+'Sources &amp; Checks'!$B$7+'Sources &amp; Checks'!$B$24</f>
-        <v>26710.7</v>
+        <f aca="false">J8-'Sources &amp; Checks'!$B$6+'Sources &amp; Checks'!$B$7</f>
+        <v>26599.5</v>
       </c>
       <c r="M8" s="94"/>
       <c r="N8" s="98" t="n">
@@ -7272,28 +7247,28 @@
       <c r="S8" s="94"/>
       <c r="T8" s="99" t="n">
         <f aca="false">L8/DCF!M22</f>
-        <v>8.56057304018973</v>
+        <v>8.52493429908339</v>
       </c>
       <c r="U8" s="99" t="n">
         <f aca="false">L8/DCF!N22</f>
-        <v>9.63450440051941</v>
+        <v>9.59439474823258</v>
       </c>
       <c r="V8" s="94"/>
       <c r="W8" s="100" t="n">
         <f aca="false">L8/DCF!M20</f>
-        <v>1.98684151802318</v>
+        <v>1.97857004715929</v>
       </c>
       <c r="X8" s="100" t="n">
         <f aca="false">L8/DCF!N20</f>
-        <v>1.91495142846901</v>
+        <v>1.90697924508012</v>
       </c>
       <c r="Y8" s="101" t="n">
         <f aca="false">L8/DCF!M23</f>
-        <v>12.9619546755957</v>
+        <v>12.9079924297569</v>
       </c>
       <c r="Z8" s="101" t="n">
         <f aca="false">L8/DCF!N23</f>
-        <v>17.1442233632863</v>
+        <v>17.0728498074454</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7323,11 +7298,11 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="107" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C10" s="102"/>
       <c r="D10" s="108" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="E10" s="108"/>
       <c r="F10" s="108"/>
@@ -7380,11 +7355,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="107" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C11" s="102"/>
       <c r="D11" s="108" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E11" s="108"/>
       <c r="F11" s="108"/>
@@ -7437,11 +7412,11 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="107" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C12" s="102"/>
       <c r="D12" s="108" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E12" s="108"/>
       <c r="F12" s="108"/>
@@ -7494,11 +7469,11 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="107" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C13" s="102"/>
       <c r="D13" s="108" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E13" s="108"/>
       <c r="F13" s="108"/>
@@ -7551,11 +7526,11 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="107" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C14" s="102"/>
       <c r="D14" s="108" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E14" s="108"/>
       <c r="F14" s="108"/>
@@ -7714,7 +7689,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="117" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C20" s="118"/>
       <c r="D20" s="118"/>
@@ -7782,7 +7757,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="117" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C21" s="118"/>
       <c r="D21" s="118"/>
@@ -7850,7 +7825,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="123" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C24" s="61"/>
       <c r="D24" s="61"/>
@@ -7863,36 +7838,36 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="87" t="s">
+        <v>126</v>
+      </c>
+      <c r="C25" s="87" t="s">
+        <v>127</v>
+      </c>
+      <c r="D25" s="87" t="s">
+        <v>128</v>
+      </c>
+      <c r="E25" s="87" t="s">
         <v>129</v>
-      </c>
-      <c r="C25" s="87" t="s">
-        <v>130</v>
-      </c>
-      <c r="D25" s="87" t="s">
-        <v>131</v>
-      </c>
-      <c r="E25" s="87" t="s">
-        <v>132</v>
       </c>
       <c r="F25" s="87" t="s">
         <v>54</v>
       </c>
       <c r="G25" s="87" t="s">
+        <v>130</v>
+      </c>
+      <c r="H25" s="87" t="s">
+        <v>131</v>
+      </c>
+      <c r="I25" s="87" t="s">
+        <v>132</v>
+      </c>
+      <c r="J25" s="87" t="s">
         <v>133</v>
-      </c>
-      <c r="H25" s="87" t="s">
-        <v>134</v>
-      </c>
-      <c r="I25" s="87" t="s">
-        <v>135</v>
-      </c>
-      <c r="J25" s="87" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="124" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C26" s="125" t="n">
         <f aca="false">U21</f>
@@ -7911,25 +7886,25 @@
         <v>2400</v>
       </c>
       <c r="G26" s="126" t="n">
-        <f aca="false">'Sources &amp; Checks'!$B$7+'Sources &amp; Checks'!$B$24</f>
-        <v>1611.2</v>
+        <f aca="false">'Sources &amp; Checks'!$B$7</f>
+        <v>1500</v>
       </c>
       <c r="H26" s="126" t="n">
         <f aca="false">E26+F26-G26</f>
-        <v>9931.62721410713</v>
+        <v>10042.8272141071</v>
       </c>
       <c r="I26" s="127" t="n">
         <f aca="false">H26/'Sources &amp; Checks'!$B$9</f>
-        <v>9.30973679612592</v>
+        <v>9.41397376650462</v>
       </c>
       <c r="J26" s="128" t="n">
         <f aca="false">I26/'Sources &amp; Checks'!$B$5-1</f>
-        <v>-0.644530859254451</v>
+        <v>-0.640550829839457</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="129" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C27" s="130" t="n">
         <f aca="false">X21</f>
@@ -7948,25 +7923,25 @@
         <v>2400</v>
       </c>
       <c r="G27" s="131" t="n">
-        <f aca="false">'Sources &amp; Checks'!$B$7+'Sources &amp; Checks'!$B$24</f>
-        <v>1611.2</v>
+        <f aca="false">'Sources &amp; Checks'!$B$7</f>
+        <v>1500</v>
       </c>
       <c r="H27" s="131" t="n">
         <f aca="false">E27+F27-G27</f>
-        <v>7052.01009167362</v>
+        <v>7163.21009167361</v>
       </c>
       <c r="I27" s="132" t="n">
         <f aca="false">H27/'Sources &amp; Checks'!$B$9</f>
-        <v>6.61043315679941</v>
+        <v>6.71467012717812</v>
       </c>
       <c r="J27" s="133" t="n">
         <f aca="false">I27/'Sources &amp; Checks'!$B$5-1</f>
-        <v>-0.747597053959549</v>
+        <v>-0.743617024544555</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="124" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C28" s="125" t="n">
         <f aca="false">Z21</f>
@@ -7985,25 +7960,25 @@
         <v>2400</v>
       </c>
       <c r="G28" s="126" t="n">
-        <f aca="false">'Sources &amp; Checks'!$B$7+'Sources &amp; Checks'!$B$24</f>
-        <v>1611.2</v>
+        <f aca="false">'Sources &amp; Checks'!$B$7</f>
+        <v>1500</v>
       </c>
       <c r="H28" s="126" t="n">
         <f aca="false">E28+F28-G28</f>
-        <v>8560.2598</v>
+        <v>8671.4598</v>
       </c>
       <c r="I28" s="127" t="n">
         <f aca="false">H28/'Sources &amp; Checks'!$B$9</f>
-        <v>8.02424053243345</v>
+        <v>8.12847750281215</v>
       </c>
       <c r="J28" s="128" t="n">
         <f aca="false">I28/'Sources &amp; Checks'!$B$5-1</f>
-        <v>-0.693614336295019</v>
+        <v>-0.689634306880025</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="134" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -8050,12 +8025,12 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="8" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="8" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8075,7 +8050,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F8" s="54" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$8*'Sources &amp; Checks'!$B$5</f>
@@ -8084,7 +8059,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="8" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F9" s="27" t="n">
         <f aca="false">F8/(F8+F15)</f>
@@ -8093,7 +8068,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F10" s="136" t="n">
         <f aca="false">F11+F14*F13</f>
@@ -8102,7 +8077,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="F11" s="37" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$10</f>
@@ -8111,7 +8086,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="8" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F12" s="137" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$11</f>
@@ -8120,7 +8095,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="8" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="F13" s="37" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$12</f>
@@ -8129,7 +8104,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="F14" s="138" t="n">
         <f aca="false">1/3*1+2/3*F12</f>
@@ -8141,7 +8116,7 @@
         <v>10</v>
       </c>
       <c r="B15" s="74" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="F15" s="139" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$7</f>
@@ -8150,7 +8125,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="8" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="F16" s="38" t="n">
         <f aca="false">F15/(F15+F8)</f>
@@ -8159,7 +8134,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="8" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="F17" s="38" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$13</f>
@@ -8168,7 +8143,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="F18" s="38" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$14</f>
@@ -8180,7 +8155,7 @@
         <v>10</v>
       </c>
       <c r="B20" s="74" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="F20" s="54" t="n">
         <f aca="false">F15+F8</f>
@@ -8227,7 +8202,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="141" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B1" s="141"/>
       <c r="C1" s="141"/>
@@ -8235,156 +8210,156 @@
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="87" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B3" s="87" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C3" s="87" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D3" s="87" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="142" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B4" s="143" t="n">
         <v>46087</v>
       </c>
       <c r="C4" s="142" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D4" s="142" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="142" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B5" s="144" t="n">
         <v>26.19</v>
       </c>
       <c r="C5" s="142" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D5" s="142" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="142" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B6" s="145" t="n">
         <v>2400</v>
       </c>
       <c r="C6" s="142" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D6" s="142" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="142" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B7" s="145" t="n">
         <v>1500</v>
       </c>
       <c r="C7" s="142" t="s">
+        <v>162</v>
+      </c>
+      <c r="D7" s="142" t="s">
         <v>165</v>
-      </c>
-      <c r="D7" s="142" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="142" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B8" s="145" t="n">
         <v>1050</v>
       </c>
       <c r="C8" s="142" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D8" s="142" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="142" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B9" s="145" t="n">
         <v>1066.8</v>
       </c>
       <c r="C9" s="142" t="s">
+        <v>167</v>
+      </c>
+      <c r="D9" s="142" t="s">
         <v>170</v>
-      </c>
-      <c r="D9" s="142" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="142" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B10" s="146" t="n">
         <v>0.028643</v>
       </c>
       <c r="C10" s="142" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D10" s="142" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="142" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B11" s="147" t="n">
         <v>1.01</v>
       </c>
       <c r="C11" s="142" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="D11" s="142" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="142" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B12" s="146" t="n">
         <v>0.06</v>
       </c>
       <c r="C12" s="142" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D12" s="142" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="142" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B13" s="146" t="n">
         <v>0.03</v>
       </c>
       <c r="C13" s="142" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D13" s="142" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8395,124 +8370,110 @@
         <v>0.12</v>
       </c>
       <c r="C14" s="142" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D14" s="142" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="148" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B16" s="148" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="148" t="s">
+        <v>182</v>
+      </c>
+      <c r="B18" s="148" t="s">
+        <v>183</v>
+      </c>
+      <c r="C18" s="148" t="s">
+        <v>184</v>
+      </c>
+      <c r="D18" s="148" t="s">
         <v>185</v>
-      </c>
-      <c r="B18" s="148" t="s">
-        <v>186</v>
-      </c>
-      <c r="C18" s="148" t="s">
-        <v>187</v>
-      </c>
-      <c r="D18" s="148" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="148" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B19" s="149" t="n">
         <v>0.0909</v>
       </c>
       <c r="C19" s="148" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D19" s="148" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="148" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B20" s="149" t="n">
         <v>0.1722</v>
       </c>
       <c r="C20" s="148" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D20" s="148" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="148" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B21" s="149" t="n">
         <v>0.0805</v>
       </c>
       <c r="C21" s="148" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D21" s="148" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="148" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B22" s="149" t="n">
         <v>0.1828</v>
       </c>
       <c r="C22" s="148" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D22" s="148" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="148" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B23" s="149" t="n">
         <v>-0.0287</v>
       </c>
       <c r="C23" s="148" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D23" s="148" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="142" t="s">
-        <v>199</v>
-      </c>
-      <c r="B24" s="145" t="n">
-        <v>111.2</v>
-      </c>
-      <c r="C24" s="142" t="s">
-        <v>165</v>
-      </c>
-      <c r="D24" s="142" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="150" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="B25" s="151" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>
@@ -8550,21 +8511,21 @@
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="154" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="C3" s="155" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="D3" s="156" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="E3" s="157" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="158" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C4" s="159" t="n">
         <v>10775</v>
@@ -8578,7 +8539,7 @@
     </row>
     <row r="5" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="162" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C5" s="163" t="n">
         <v>9332</v>
@@ -8592,7 +8553,7 @@
     </row>
     <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="162" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C6" s="163" t="n">
         <v>1443</v>
@@ -8606,7 +8567,7 @@
     </row>
     <row r="7" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="166" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C7" s="167" t="n">
         <v>1314</v>
@@ -8620,21 +8581,21 @@
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="154" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C10" s="155" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="D10" s="156" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="E10" s="157" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="158" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C11" s="159" t="n">
         <v>16406</v>
@@ -8648,7 +8609,7 @@
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="162" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C12" s="163" t="n">
         <v>5643</v>
@@ -8662,7 +8623,7 @@
     </row>
     <row r="13" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="166" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C13" s="167" t="n">
         <v>4675</v>
@@ -8676,21 +8637,21 @@
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="154" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C16" s="155" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="D16" s="156" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="E16" s="157" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="158" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="C17" s="159" t="n">
         <v>7422</v>
@@ -8704,7 +8665,7 @@
     </row>
     <row r="18" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="162" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="C18" s="163" t="n">
         <v>3341</v>
@@ -8718,7 +8679,7 @@
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="170" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="C19" s="171" t="n">
         <f aca="false">C17+C18</f>
@@ -8735,21 +8696,21 @@
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="154" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="C22" s="155" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="D22" s="156" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="E22" s="157" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="158" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="C23" s="174" t="n">
         <f aca="false">(C4-4800.9)/4800.9</f>
@@ -8766,10 +8727,10 @@
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="162" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C24" s="176" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="D24" s="177" t="n">
         <f aca="false">(D7-C7)/C7</f>
@@ -8782,7 +8743,7 @@
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="162" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="C25" s="179" t="n">
         <f aca="false">C7/C4</f>
@@ -8799,7 +8760,7 @@
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="162" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="C26" s="179" t="n">
         <f aca="false">(C4-C5)/C4</f>
@@ -8816,7 +8777,7 @@
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="162" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C27" s="179" t="n">
         <f aca="false">C5/C4</f>
@@ -8833,7 +8794,7 @@
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="162" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="C28" s="179" t="n">
         <f aca="false">C7/C11</f>
@@ -8850,7 +8811,7 @@
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="162" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="C29" s="179" t="n">
         <f aca="false">C7/C12</f>
@@ -8867,7 +8828,7 @@
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="162" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="C30" s="179" t="n">
         <f aca="false">C19/C11</f>
@@ -8884,7 +8845,7 @@
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="166" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="C31" s="180" t="n">
         <f aca="false">C12/C11</f>
@@ -8901,17 +8862,17 @@
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="152" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="152" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="152" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>
@@ -8943,12 +8904,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="80" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="81" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="C3" s="81"/>
     </row>
@@ -8963,7 +8924,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="83" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="C5" s="184" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$21</f>
@@ -8972,7 +8933,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="83" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="C6" s="184" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$22</f>
@@ -8981,7 +8942,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="83" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="C7" s="184" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$23</f>
@@ -8990,7 +8951,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="83" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="C8" s="185" t="n">
         <f aca="false">DCF!$N$20</f>
@@ -8999,7 +8960,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="83" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="C9" s="185" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$6</f>
@@ -9008,16 +8969,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="83" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="C10" s="185" t="n">
-        <f aca="false">'Sources &amp; Checks'!$B$7+'Sources &amp; Checks'!$B$24</f>
-        <v>1611.2</v>
+        <f aca="false">'Sources &amp; Checks'!$B$7</f>
+        <v>1500</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="83" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C11" s="185" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$9</f>
@@ -9035,7 +8996,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="187" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9059,13 +9020,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="188" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="C16" s="188" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E16" s="188" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F16" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -9113,7 +9074,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="83" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C17" s="184" t="n">
         <f aca="false">DCF!$H$11</f>
@@ -9165,7 +9126,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="83" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C18" s="184" t="n">
         <f aca="false">DCF!$H$13</f>
@@ -9224,7 +9185,7 @@
         <v>0.092</v>
       </c>
       <c r="E19" s="83" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="F19" s="191" t="n">
         <f aca="false">F18*$C$18*(1-$C$4)</f>
@@ -9273,7 +9234,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="83" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C20" s="184" t="n">
         <f aca="false">DCF!$H$17</f>
@@ -9378,7 +9339,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E22" s="83" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="F22" s="191" t="n">
         <f aca="false">F19*F21</f>
@@ -9472,14 +9433,14 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="83" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="C24" s="185" t="n">
         <f aca="false">SUM(F25:O25)</f>
         <v>10677.2345379775</v>
       </c>
       <c r="E24" s="83" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="F24" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -9531,7 +9492,7 @@
         <v>31861.0982339967</v>
       </c>
       <c r="E25" s="83" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="F25" s="191" t="n">
         <f aca="false">F23*DCF!$O$70/(1+$C$19)^F24</f>
@@ -9576,7 +9537,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="83" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C26" s="185" t="n">
         <f aca="false">C25/(1+$C$19)^O24</f>
@@ -9585,7 +9546,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="83" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C27" s="185" t="n">
         <f aca="false">C24+C26</f>
@@ -9594,25 +9555,25 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="83" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C28" s="185" t="n">
         <f aca="false">C27+$C$9-$C$10</f>
-        <v>26453.0089420393</v>
+        <v>26564.2089420393</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="188" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="C29" s="196" t="n">
         <f aca="false">C28/$C$11</f>
-        <v>24.7965963086233</v>
+        <v>24.900833279002</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="83" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C30" s="183" t="n">
         <f aca="false">1-P23/P19</f>
@@ -9621,7 +9582,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="83" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C31" s="183" t="n">
         <f aca="false">C26/C27</f>
@@ -9649,13 +9610,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="188" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="C35" s="188" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E35" s="188" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F35" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -9703,7 +9664,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="83" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C36" s="184" t="n">
         <f aca="false">DCF!$L$11</f>
@@ -9755,7 +9716,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="83" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C37" s="184" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -9814,7 +9775,7 @@
         <v>0.0858027889618787</v>
       </c>
       <c r="E38" s="83" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="F38" s="191" t="n">
         <f aca="false">F37*$C$37*(1-$C$4)</f>
@@ -9863,7 +9824,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="83" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C39" s="184" t="n">
         <f aca="false">DCF!$L$17</f>
@@ -9968,7 +9929,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E41" s="83" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="F41" s="191" t="n">
         <f aca="false">F38*F40</f>
@@ -10062,14 +10023,14 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="83" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="C43" s="185" t="n">
         <f aca="false">SUM(F44:O44)</f>
         <v>12309.8454096608</v>
       </c>
       <c r="E43" s="83" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="F43" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -10121,7 +10082,7 @@
         <v>41776.8531981022</v>
       </c>
       <c r="E44" s="83" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="F44" s="191" t="n">
         <f aca="false">F42*DCF!$O$70/(1+$C$38)^F43</f>
@@ -10166,7 +10127,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="83" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C45" s="185" t="n">
         <f aca="false">C44/(1+$C$38)^O43</f>
@@ -10175,7 +10136,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="83" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C46" s="185" t="n">
         <f aca="false">C43+C45</f>
@@ -10184,25 +10145,25 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="83" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C47" s="185" t="n">
         <f aca="false">C46+$C$9-$C$10</f>
-        <v>33732.0037132682</v>
+        <v>33843.2037132682</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="188" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="C48" s="196" t="n">
         <f aca="false">C47/$C$11</f>
-        <v>31.6198010060632</v>
+        <v>31.7240379764419</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="83" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C49" s="183" t="n">
         <f aca="false">1-P42/P38</f>
@@ -10211,7 +10172,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="83" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C50" s="183" t="n">
         <f aca="false">C45/C46</f>
@@ -10239,13 +10200,13 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="188" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="C54" s="188" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E54" s="188" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F54" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -10293,7 +10254,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="83" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C55" s="184" t="n">
         <f aca="false">DCF!$P$11</f>
@@ -10345,7 +10306,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="83" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C56" s="184" t="n">
         <f aca="false">DCF!$P$13</f>
@@ -10404,7 +10365,7 @@
         <v>0.082</v>
       </c>
       <c r="E57" s="83" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="F57" s="191" t="n">
         <f aca="false">F56*$C$56*(1-$C$4)</f>
@@ -10453,7 +10414,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="83" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C58" s="184" t="n">
         <f aca="false">DCF!$P$17</f>
@@ -10558,7 +10519,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E60" s="83" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="F60" s="191" t="n">
         <f aca="false">F57*F59</f>
@@ -10652,14 +10613,14 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B62" s="83" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="C62" s="185" t="n">
         <f aca="false">SUM(F63:O63)</f>
         <v>14171.7844838877</v>
       </c>
       <c r="E62" s="83" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="F62" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -10711,7 +10672,7 @@
         <v>52830.3906260597</v>
       </c>
       <c r="E63" s="83" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="F63" s="191" t="n">
         <f aca="false">F61*DCF!$O$70/(1+$C$57)^F62</f>
@@ -10756,7 +10717,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="83" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C64" s="185" t="n">
         <f aca="false">C63/(1+$C$57)^O62</f>
@@ -10765,7 +10726,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="83" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C65" s="185" t="n">
         <f aca="false">C62+C64</f>
@@ -10774,25 +10735,25 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B66" s="83" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C66" s="185" t="n">
         <f aca="false">C65+$C$9-$C$10</f>
-        <v>41849.6192212229</v>
+        <v>41960.8192212229</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B67" s="188" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="C67" s="196" t="n">
         <f aca="false">C66/$C$11</f>
-        <v>39.2291143805989</v>
+        <v>39.3333513509776</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B68" s="83" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C68" s="183" t="n">
         <f aca="false">1-P61/P57</f>
@@ -10801,7 +10762,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B69" s="83" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C69" s="183" t="n">
         <f aca="false">C64/C65</f>
@@ -10810,12 +10771,12 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B72" s="187" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B73" s="81" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="C73" s="81"/>
       <c r="D73" s="81"/>
@@ -10834,13 +10795,13 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B74" s="188" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="C74" s="188" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E74" s="188" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F74" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -10888,7 +10849,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B75" s="83" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C75" s="184" t="n">
         <f aca="false">DCF!$L$11</f>
@@ -10940,7 +10901,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B76" s="83" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C76" s="184" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -10999,7 +10960,7 @@
         <v>0.0858027889618787</v>
       </c>
       <c r="E77" s="83" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="F77" s="191" t="n">
         <f aca="false">F76*$C$76*(1-$C$4)</f>
@@ -11048,7 +11009,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B78" s="83" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C78" s="184" t="n">
         <f aca="false">DCF!$D$92</f>
@@ -11153,7 +11114,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E80" s="83" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="F80" s="191" t="n">
         <f aca="false">F77*F79</f>
@@ -11247,14 +11208,14 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B82" s="83" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="C82" s="185" t="n">
         <f aca="false">SUM(F83:O83)</f>
         <v>12935.2230595844</v>
       </c>
       <c r="E82" s="83" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="F82" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -11306,7 +11267,7 @@
         <v>39411.8359558047</v>
       </c>
       <c r="E83" s="83" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="F83" s="191" t="n">
         <f aca="false">F81*DCF!$O$70/(1+$C$77)^F82</f>
@@ -11351,7 +11312,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B84" s="83" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C84" s="185" t="n">
         <f aca="false">C83/(1+$C$77)^O82</f>
@@ -11360,7 +11321,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B85" s="83" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C85" s="185" t="n">
         <f aca="false">C82+C84</f>
@@ -11369,25 +11330,25 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B86" s="83" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C86" s="185" t="n">
         <f aca="false">C85+$C$9-$C$10</f>
-        <v>33189.3123388655</v>
+        <v>33300.5123388655</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B87" s="188" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="C87" s="196" t="n">
         <f aca="false">C86/$C$11</f>
-        <v>31.1110914312575</v>
+        <v>31.2153284016362</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B88" s="83" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C88" s="183" t="n">
         <f aca="false">1-P81/P77</f>
@@ -11396,7 +11357,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B89" s="83" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C89" s="183" t="n">
         <f aca="false">C84/C85</f>
@@ -11405,7 +11366,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B92" s="81" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="C92" s="81"/>
       <c r="D92" s="81"/>
@@ -11424,13 +11385,13 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B93" s="188" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="C93" s="188" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E93" s="188" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F93" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -11478,7 +11439,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B94" s="83" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C94" s="184" t="n">
         <f aca="false">DCF!$L$11</f>
@@ -11530,7 +11491,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B95" s="83" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C95" s="184" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -11589,7 +11550,7 @@
         <v>0.0858027889618787</v>
       </c>
       <c r="E96" s="83" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="F96" s="191" t="n">
         <f aca="false">F95*$C$95*(1-$C$4)</f>
@@ -11638,7 +11599,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B97" s="83" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C97" s="184" t="n">
         <f aca="false">DCF!$F$92</f>
@@ -11743,7 +11704,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E99" s="83" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="F99" s="191" t="n">
         <f aca="false">F96*F98</f>
@@ -11837,14 +11798,14 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B101" s="83" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="C101" s="185" t="n">
         <f aca="false">SUM(F102:O102)</f>
         <v>12628.0179564231</v>
       </c>
       <c r="E101" s="83" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="F101" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -11896,7 +11857,7 @@
         <v>40579.3082501446</v>
       </c>
       <c r="E102" s="83" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="F102" s="191" t="n">
         <f aca="false">F100*DCF!$O$70/(1+$C$96)^F101</f>
@@ -11941,7 +11902,7 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B103" s="83" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C103" s="185" t="n">
         <f aca="false">C102/(1+$C$96)^O101</f>
@@ -11950,7 +11911,7 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B104" s="83" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C104" s="185" t="n">
         <f aca="false">C101+C103</f>
@@ -11959,25 +11920,25 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B105" s="83" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C105" s="185" t="n">
         <f aca="false">C104+$C$9-$C$10</f>
-        <v>33458.7153886549</v>
+        <v>33569.9153886549</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B106" s="188" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="C106" s="196" t="n">
         <f aca="false">C105/$C$11</f>
-        <v>31.363625223711</v>
+        <v>31.4678621940897</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B107" s="83" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C107" s="183" t="n">
         <f aca="false">1-P100/P96</f>
@@ -11986,7 +11947,7 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B108" s="83" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C108" s="183" t="n">
         <f aca="false">C103/C104</f>
@@ -11995,7 +11956,7 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B111" s="81" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="C111" s="81"/>
       <c r="D111" s="81"/>
@@ -12014,13 +11975,13 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B112" s="188" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="C112" s="188" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E112" s="188" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F112" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -12068,7 +12029,7 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B113" s="83" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C113" s="184" t="n">
         <f aca="false">DCF!$L$11</f>
@@ -12120,7 +12081,7 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B114" s="83" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C114" s="184" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -12179,7 +12140,7 @@
         <v>0.0858027889618787</v>
       </c>
       <c r="E115" s="83" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="F115" s="191" t="n">
         <f aca="false">F114*$C$114*(1-$C$4)</f>
@@ -12228,7 +12189,7 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B116" s="83" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C116" s="184" t="n">
         <f aca="false">DCF!$H$92</f>
@@ -12333,7 +12294,7 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E118" s="83" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="F118" s="191" t="n">
         <f aca="false">F115*F117</f>
@@ -12427,14 +12388,14 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B120" s="83" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="C120" s="185" t="n">
         <f aca="false">SUM(F121:O121)</f>
         <v>12309.8454096608</v>
       </c>
       <c r="E120" s="83" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="F120" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -12486,7 +12447,7 @@
         <v>41776.8531981022</v>
       </c>
       <c r="E121" s="83" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="F121" s="191" t="n">
         <f aca="false">F119*DCF!$O$70/(1+$C$115)^F120</f>
@@ -12531,7 +12492,7 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B122" s="83" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C122" s="185" t="n">
         <f aca="false">C121/(1+$C$115)^O120</f>
@@ -12540,7 +12501,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B123" s="83" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C123" s="185" t="n">
         <f aca="false">C120+C122</f>
@@ -12549,25 +12510,25 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B124" s="83" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C124" s="185" t="n">
         <f aca="false">C123+$C$9-$C$10</f>
-        <v>33732.0037132682</v>
+        <v>33843.2037132682</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B125" s="188" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="C125" s="196" t="n">
         <f aca="false">C124/$C$11</f>
-        <v>31.6198010060632</v>
+        <v>31.7240379764419</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B126" s="83" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C126" s="183" t="n">
         <f aca="false">1-P119/P115</f>
@@ -12576,7 +12537,7 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B127" s="83" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C127" s="183" t="n">
         <f aca="false">C122/C123</f>
@@ -12585,7 +12546,7 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B130" s="81" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C130" s="81"/>
       <c r="D130" s="81"/>
@@ -12604,13 +12565,13 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B131" s="188" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="C131" s="188" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E131" s="188" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F131" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -12658,7 +12619,7 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B132" s="83" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C132" s="184" t="n">
         <f aca="false">DCF!$L$11</f>
@@ -12710,7 +12671,7 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B133" s="83" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C133" s="184" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -12769,7 +12730,7 @@
         <v>0.0858027889618787</v>
       </c>
       <c r="E134" s="83" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="F134" s="191" t="n">
         <f aca="false">F133*$C$133*(1-$C$4)</f>
@@ -12818,7 +12779,7 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B135" s="83" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C135" s="184" t="n">
         <f aca="false">DCF!$J$92</f>
@@ -12923,7 +12884,7 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E137" s="83" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="F137" s="191" t="n">
         <f aca="false">F134*F136</f>
@@ -13017,14 +12978,14 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B139" s="83" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="C139" s="185" t="n">
         <f aca="false">SUM(F140:O140)</f>
         <v>11980.4344599675</v>
       </c>
       <c r="E139" s="83" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="F139" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -13076,7 +13037,7 @@
         <v>43005.1340184788</v>
       </c>
       <c r="E140" s="83" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="F140" s="191" t="n">
         <f aca="false">F138*DCF!$O$70/(1+$C$134)^F139</f>
@@ -13121,7 +13082,7 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B141" s="83" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C141" s="185" t="n">
         <f aca="false">C140/(1+$C$134)^O139</f>
@@ -13130,7 +13091,7 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B142" s="83" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C142" s="185" t="n">
         <f aca="false">C139+C141</f>
@@ -13139,25 +13100,25 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B143" s="83" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C143" s="185" t="n">
         <f aca="false">C142+$C$9-$C$10</f>
-        <v>34009.2339134984</v>
+        <v>34120.4339134984</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B144" s="188" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="C144" s="196" t="n">
         <f aca="false">C143/$C$11</f>
-        <v>31.8796718349254</v>
+        <v>31.9839088053041</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B145" s="83" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C145" s="183" t="n">
         <f aca="false">1-P138/P134</f>
@@ -13166,7 +13127,7 @@
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B146" s="83" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C146" s="183" t="n">
         <f aca="false">C141/C142</f>
@@ -13175,7 +13136,7 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B149" s="81" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="C149" s="81"/>
       <c r="D149" s="81"/>
@@ -13194,13 +13155,13 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B150" s="188" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="C150" s="188" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E150" s="188" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F150" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -13248,7 +13209,7 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B151" s="83" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C151" s="184" t="n">
         <f aca="false">DCF!$L$11</f>
@@ -13300,7 +13261,7 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B152" s="83" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C152" s="184" t="n">
         <f aca="false">DCF!$L$13</f>
@@ -13359,7 +13320,7 @@
         <v>0.0858027889618787</v>
       </c>
       <c r="E153" s="83" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="F153" s="191" t="n">
         <f aca="false">F152*$C$152*(1-$C$4)</f>
@@ -13408,7 +13369,7 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B154" s="83" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C154" s="184" t="n">
         <f aca="false">DCF!$L$92</f>
@@ -13513,7 +13474,7 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E156" s="83" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="F156" s="191" t="n">
         <f aca="false">F153*F155</f>
@@ -13607,14 +13568,14 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B158" s="83" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="C158" s="185" t="n">
         <f aca="false">SUM(F159:O159)</f>
         <v>11639.5088061378</v>
       </c>
       <c r="E158" s="83" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="F158" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -13666,7 +13627,7 @@
         <v>44264.8262118657</v>
       </c>
       <c r="E159" s="83" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="F159" s="191" t="n">
         <f aca="false">F157*DCF!$O$70/(1+$C$153)^F158</f>
@@ -13711,7 +13672,7 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B160" s="83" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C160" s="185" t="n">
         <f aca="false">C159/(1+$C$153)^O158</f>
@@ -13720,7 +13681,7 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B161" s="83" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C161" s="185" t="n">
         <f aca="false">C158+C160</f>
@@ -13729,25 +13690,25 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B162" s="83" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C162" s="185" t="n">
         <f aca="false">C161+$C$9-$C$10</f>
-        <v>34290.4633141712</v>
+        <v>34401.6633141712</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B163" s="188" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="C163" s="196" t="n">
         <f aca="false">C162/$C$11</f>
-        <v>32.1432914456048</v>
+        <v>32.2475284159835</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B164" s="83" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C164" s="183" t="n">
         <f aca="false">1-P157/P153</f>
@@ -13756,7 +13717,7 @@
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B165" s="83" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C165" s="183" t="n">
         <f aca="false">C160/C161</f>

</xml_diff>

<commit_message>
Remove leftover cell references and placeholders
</commit_message>
<xml_diff>
--- a/Ryanair_DCF_Model_Kodickova_2026.xlsx
+++ b/Ryanair_DCF_Model_Kodickova_2026.xlsx
@@ -460,7 +460,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="247">
   <si>
     <t xml:space="preserve">DCF Model - Ryanair</t>
   </si>
@@ -474,18 +474,12 @@
     <t xml:space="preserve">Implied Price Per Share</t>
   </si>
   <si>
-    <t xml:space="preserve">Low-end</t>
-  </si>
-  <si>
     <t xml:space="preserve">Date</t>
   </si>
   <si>
     <t xml:space="preserve">Current Share Price</t>
   </si>
   <si>
-    <t xml:space="preserve">High-end</t>
-  </si>
-  <si>
     <t xml:space="preserve">Year end</t>
   </si>
   <si>
@@ -534,7 +528,7 @@
     <t xml:space="preserve">TGR</t>
   </si>
   <si>
-    <t xml:space="preserve">D&amp;A 8.0% | CapEx 18.3% | WC -2.9%</t>
+    <t xml:space="preserve">FY26: D&amp;A 8.0% | CapEx 18.3% | WC -2.9%</t>
   </si>
   <si>
     <t xml:space="preserve">Normalized avg</t>
@@ -639,7 +633,7 @@
     <t xml:space="preserve">Implied Stock Price</t>
   </si>
   <si>
-    <t xml:space="preserve">Scenario Analysis — Implied Share Price (€)</t>
+    <t xml:space="preserve">Scenario Analysis - Implied Share Price (€)</t>
   </si>
   <si>
     <t xml:space="preserve">Scenario</t>
@@ -678,51 +672,33 @@
     <t xml:space="preserve">Cost of equity</t>
   </si>
   <si>
-    <t xml:space="preserve">WACC!F14, F10</t>
-  </si>
-  <si>
     <t xml:space="preserve">Blume adjusted beta = 1/3 x 1 + 2/3 x raw beta, used in the cost of equity.</t>
   </si>
   <si>
     <t xml:space="preserve">Revenue growth</t>
   </si>
   <si>
-    <t xml:space="preserve">DCF!P41:X43, D18</t>
-  </si>
-  <si>
     <t xml:space="preserve">FY26 growth is the scenario rate. From FY27 growth falls by (start growth - TGR) / 9 a year, so FY35 growth equals the terminal growth rate.</t>
   </si>
   <si>
     <t xml:space="preserve">Reinvestment</t>
   </si>
   <si>
-    <t xml:space="preserve">DCF!P60:X65</t>
-  </si>
-  <si>
     <t xml:space="preserve">Reinvestment rate = growth / RONIC. FY26 is implied by the CapEx, D&amp;A and working capital assumptions. From FY27 RONIC fades in equal steps to WACC in FY35. CapEx and working capital follow it.</t>
   </si>
   <si>
     <t xml:space="preserve">Terminal value</t>
   </si>
   <si>
-    <t xml:space="preserve">DCF!Y54:Y66, X73</t>
-  </si>
-  <si>
     <t xml:space="preserve">Terminal FCF = NOPAT FY35 x (1+g) x (1 - g/WACC), TV = terminal FCF / (WACC - g). RONIC = WACC, so the terminal year continues the FY35 reinvestment rate.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sources &amp; Checks!B14</t>
-  </si>
-  <si>
     <t xml:space="preserve">Effective tax rate of 12%, as reported in the Q3 FY26 results (note 4).</t>
   </si>
   <si>
     <t xml:space="preserve">FY26 cash flow</t>
   </si>
   <si>
-    <t xml:space="preserve">DCF!O67</t>
-  </si>
-  <si>
     <t xml:space="preserve">Only the 25 days between the valuation date and the FY26 year end are counted.</t>
   </si>
   <si>
@@ -1017,7 +993,7 @@
     <t xml:space="preserve">-</t>
   </si>
   <si>
-    <t xml:space="preserve">All forecast drivers (revenue growth, EBIT margin, D&amp;A, CapEx, ΔWC) use flat normalized avg. Normal years: FY2017-2019 + FY2024-2025. Excluded: FY2020-2023 (Covid disruption + rebound distortion). Revenue growth starts at the normalised rate in FY26 and fades in equal steps to the terminal growth rate by FY35. From FY27 the reinvestment rate equals growth / RONIC, with RONIC fading from its FY26 implied level to WACC.</t>
+    <t xml:space="preserve">Starting levels use the normalised average of FY2017-2019 and FY2024-2025 (FY2020-2023 excluded for Covid disruption and rebound). Revenue growth starts at the normalised rate in FY26 and fades in equal steps to the terminal growth rate by FY35. EBIT margin is held flat. From FY27 the reinvestment rate equals growth / RONIC, with RONIC fading from its FY26 implied level to WACC.</t>
   </si>
   <si>
     <t xml:space="preserve">Normalized Revenue Growth</t>
@@ -1050,10 +1026,10 @@
     <t xml:space="preserve">Avg of FY17-FY19 + FY24-FY25 change in net working capital as % of Revenue (negative = cash source, typical for airlines)</t>
   </si>
   <si>
-    <t xml:space="preserve">⚠ Data Note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FY2016 historical revenue (€6,535.8M) should be verified against Ryanair's FY2016 Annual Report (year ended 31 March 2016). Some databases report FY2016 total revenues as ~€5,654M (ex-ancillary supplements). If restated, the normalized growth average would adjust from 9.09% to approx. 9.5%.</t>
+    <t xml:space="preserve">Data note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY2016 historical revenue (€6,535.8M) is taken from the database used. Some sources report FY2016 total revenues of about €5,654M (ex-ancillary supplements); if restated, the normalised growth average would adjust from 9.09% to approx. 9.5%.</t>
   </si>
   <si>
     <t xml:space="preserve">Income Statement Data (€ million)</t>
@@ -1092,6 +1068,9 @@
     <t xml:space="preserve">Gross Cash1</t>
   </si>
   <si>
+    <t xml:space="preserve">Liabilities</t>
+  </si>
+  <si>
     <t xml:space="preserve">Current Liabilities1</t>
   </si>
   <si>
@@ -1222,21 +1201,6 @@
   </si>
   <si>
     <t xml:space="preserve">Sensitivity table cash flows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sensitivity, terminal growth from DCF!D92</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sensitivity, terminal growth from DCF!F92</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sensitivity, terminal growth from DCF!H92</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sensitivity, terminal growth from DCF!J92</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sensitivity, terminal growth from DCF!L92</t>
   </si>
 </sst>
 </file>
@@ -3159,13 +3123,11 @@
         <f aca="false">S81</f>
         <v>31.7240379764419</v>
       </c>
-      <c r="K5" s="8" t="s">
-        <v>4</v>
-      </c>
+      <c r="K5" s="8"/>
     </row>
     <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="10" t="n">
@@ -3173,26 +3135,24 @@
         <v>46087</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I6" s="9" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$5</f>
         <v>26.19</v>
       </c>
-      <c r="K6" s="8" t="s">
-        <v>7</v>
-      </c>
+      <c r="K6" s="8"/>
     </row>
     <row r="7" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="11" t="n">
         <v>46112</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I7" s="12" t="n">
         <f aca="false">I5/I6-1</f>
@@ -3201,10 +3161,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C9" s="15"/>
       <c r="D9" s="15"/>
@@ -3231,40 +3191,40 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="J10" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="N10" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="N10" s="8" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D11" s="16" t="n">
         <v>2</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H11" s="17" t="n">
         <v>0.07</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L11" s="17" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$19</f>
         <v>0.0909</v>
       </c>
       <c r="N11" s="8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P11" s="17" t="n">
         <v>0.11</v>
@@ -3272,52 +3232,52 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D12" s="16" t="n">
         <v>2</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L12" s="17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="N12" s="8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="P12" s="17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D13" s="16" t="n">
         <v>2</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H13" s="17" t="n">
         <v>0.16</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="L13" s="17" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$20</f>
         <v>0.1722</v>
       </c>
       <c r="N13" s="8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="P13" s="17" t="n">
         <v>0.185</v>
@@ -3325,28 +3285,28 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D14" s="16" t="n">
         <v>2</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="L14" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="N14" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="P14" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3354,27 +3314,27 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D16" s="18" t="n">
         <f aca="false">CHOOSE(D13,H16,L16,P16)</f>
         <v>0.0858027889618787</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H16" s="19" t="n">
         <v>0.092</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="L16" s="18" t="n">
         <f aca="false">WACC!F22</f>
         <v>0.0858027889618787</v>
       </c>
       <c r="N16" s="8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="P16" s="19" t="n">
         <v>0.082</v>
@@ -3382,26 +3342,26 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D17" s="19" t="n">
         <f aca="false">CHOOSE(D14,H17,L17,P17)</f>
         <v>0.015</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H17" s="19" t="n">
         <v>0.01</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="L17" s="19" t="n">
         <v>0.015</v>
       </c>
       <c r="N17" s="8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="P17" s="19" t="n">
         <v>0.02</v>
@@ -3409,7 +3369,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D18" s="20" t="n">
         <f aca="false">COLUMNS(P40:X40)</f>
@@ -3418,10 +3378,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="21" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C19" s="15"/>
       <c r="D19" s="15"/>
@@ -3507,7 +3467,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="24" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E20" s="25" t="n">
         <v>6535.8</v>
@@ -3582,12 +3542,12 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="27" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C21" s="28"/>
       <c r="D21" s="28"/>
       <c r="E21" s="27" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F21" s="27" t="n">
         <f aca="false">F20/E20-1</f>
@@ -3668,7 +3628,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E22" s="25" t="n">
         <f aca="false">E23+E28</f>
@@ -3753,7 +3713,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="24" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E23" s="25" t="n">
         <v>1460.1</v>
@@ -3828,7 +3788,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="27" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C24" s="28"/>
       <c r="D24" s="28"/>
@@ -3915,7 +3875,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="24" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E25" s="25" t="n">
         <v>162.8</v>
@@ -3990,7 +3950,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="27" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C26" s="28"/>
       <c r="D26" s="28"/>
@@ -4077,10 +4037,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B27" s="22" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C27" s="15"/>
       <c r="D27" s="23"/>
@@ -4167,7 +4127,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="24" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E28" s="25" t="n">
         <v>427.3</v>
@@ -4242,7 +4202,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="27" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C29" s="30"/>
       <c r="D29" s="30"/>
@@ -4334,7 +4294,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E31" s="25" t="n">
         <v>1217.7</v>
@@ -4409,7 +4369,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="27" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C32" s="28"/>
       <c r="D32" s="28"/>
@@ -4496,7 +4456,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="24" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E34" s="25" t="n">
         <v>-135.6</v>
@@ -4571,7 +4531,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="27" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C35" s="30"/>
       <c r="D35" s="30"/>
@@ -4658,7 +4618,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="31" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C36" s="30"/>
       <c r="D36" s="30"/>
@@ -4702,10 +4662,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="21" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B38" s="32" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C38" s="33"/>
       <c r="D38" s="34"/>
@@ -4790,12 +4750,12 @@
         <v>2035</v>
       </c>
       <c r="Y38" s="35" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="24" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E39" s="25" t="n">
         <f aca="false">E20</f>
@@ -4880,7 +4840,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="27" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C40" s="28"/>
       <c r="D40" s="28"/>
@@ -4968,7 +4928,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="36" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="O41" s="37" t="n">
         <f aca="false">$H$11</f>
@@ -5013,7 +4973,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="36" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="O42" s="37" t="n">
         <f aca="false">$L$11</f>
@@ -5058,7 +5018,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="36" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O43" s="37" t="n">
         <f aca="false">$P$11</f>
@@ -5103,7 +5063,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="24" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E45" s="25" t="n">
         <f aca="false">E23</f>
@@ -5188,7 +5148,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="27" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C46" s="28"/>
       <c r="D46" s="28"/>
@@ -5275,7 +5235,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="36" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D47" s="28"/>
       <c r="O47" s="37" t="n">
@@ -5321,7 +5281,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="36" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D48" s="28"/>
       <c r="O48" s="37" t="n">
@@ -5367,7 +5327,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="36" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D49" s="28"/>
       <c r="O49" s="37" t="n">
@@ -5413,7 +5373,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="24" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E51" s="25" t="n">
         <f aca="false">E25</f>
@@ -5498,7 +5458,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="27" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C52" s="28"/>
       <c r="D52" s="28"/>
@@ -5585,10 +5545,10 @@
     </row>
     <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="39" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B54" s="40" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C54" s="41"/>
       <c r="D54" s="41"/>
@@ -5650,7 +5610,7 @@
     <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="24" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E56" s="25" t="n">
         <f aca="false">E28</f>
@@ -5735,7 +5695,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="27" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C57" s="30"/>
       <c r="E57" s="27" t="n">
@@ -5824,7 +5784,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B59" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E59" s="25" t="n">
         <f aca="false">E31</f>
@@ -5909,7 +5869,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B60" s="27" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C60" s="28"/>
       <c r="E60" s="27" t="n">
@@ -5995,7 +5955,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B62" s="24" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E62" s="25" t="n">
         <f aca="false">E34</f>
@@ -6080,7 +6040,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B63" s="27" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C63" s="30"/>
       <c r="E63" s="27" t="n">
@@ -6166,7 +6126,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="27" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="O64" s="43" t="n">
         <f aca="false">O40/O65</f>
@@ -6215,7 +6175,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="27" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O65" s="43" t="n">
         <f aca="false">O40/(('Sources &amp; Checks'!$B$22-'Sources &amp; Checks'!$B$21+'Sources &amp; Checks'!$B$23)/(O46*(1-O52)))</f>
@@ -6264,10 +6224,10 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="39" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B66" s="44" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C66" s="45"/>
       <c r="D66" s="45"/>
@@ -6328,7 +6288,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B67" s="47" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
@@ -6385,10 +6345,10 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="13" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B70" s="49" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="O70" s="50" t="n">
         <f aca="false">YEARFRAC(D6,D7)</f>
@@ -6397,7 +6357,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B71" s="51" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="O71" s="51" t="n">
         <f aca="false">O70/2</f>
@@ -6442,7 +6402,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B73" s="25" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="S73" s="52"/>
       <c r="T73" s="52"/>
@@ -6456,7 +6416,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B74" s="25" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="S74" s="52"/>
       <c r="T74" s="52"/>
@@ -6470,7 +6430,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B75" s="25" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="S75" s="25" t="n">
         <f aca="false">SUM(O67:X67)+X74</f>
@@ -6484,7 +6444,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B76" s="25" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="S76" s="25" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$6</f>
@@ -6498,7 +6458,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B77" s="25" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="S77" s="25" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$7</f>
@@ -6507,10 +6467,10 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="39" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B78" s="53" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="S78" s="25" t="n">
         <f aca="false">S75+S76-S77</f>
@@ -6524,7 +6484,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B80" s="54" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="S80" s="54" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$9</f>
@@ -6533,10 +6493,10 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="55" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B81" s="56" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="S81" s="57" t="n">
         <f aca="false">S78/S80</f>
@@ -6551,7 +6511,7 @@
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="59"/>
       <c r="B85" s="60" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C85" s="61"/>
       <c r="D85" s="61"/>
@@ -6568,30 +6528,30 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B86" s="62" t="s">
+        <v>58</v>
+      </c>
+      <c r="D86" s="62" t="s">
+        <v>59</v>
+      </c>
+      <c r="F86" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="D86" s="62" t="s">
+      <c r="H86" s="62" t="s">
+        <v>19</v>
+      </c>
+      <c r="J86" s="62" t="s">
+        <v>21</v>
+      </c>
+      <c r="L86" s="62" t="s">
         <v>61</v>
       </c>
-      <c r="F86" s="62" t="s">
+      <c r="N86" s="62" t="s">
         <v>62</v>
-      </c>
-      <c r="H86" s="62" t="s">
-        <v>21</v>
-      </c>
-      <c r="J86" s="62" t="s">
-        <v>23</v>
-      </c>
-      <c r="L86" s="62" t="s">
-        <v>63</v>
-      </c>
-      <c r="N86" s="62" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B87" s="63" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D87" s="64" t="n">
         <f aca="false">$H$11</f>
@@ -6620,7 +6580,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B88" s="68" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D88" s="69" t="n">
         <f aca="false">$L$11</f>
@@ -6649,7 +6609,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B89" s="63" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D89" s="64" t="n">
         <f aca="false">$P$11</f>
@@ -6678,15 +6638,15 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B90" s="73" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="59" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B91" s="74" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C91" s="61"/>
       <c r="D91" s="61"/>
@@ -6706,7 +6666,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B92" s="62" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D92" s="75" t="n">
         <v>0.005</v>
@@ -6923,90 +6883,71 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:D9"/>
+  <dimension ref="B1:C9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="130"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.43"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="80" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="81" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C3" s="81"/>
-      <c r="D3" s="81"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="82" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C4" s="83" t="s">
-        <v>72</v>
-      </c>
-      <c r="D4" s="83" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="82" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C5" s="83" t="s">
-        <v>75</v>
-      </c>
-      <c r="D5" s="83" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="82" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C6" s="83" t="s">
-        <v>78</v>
-      </c>
-      <c r="D6" s="83" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="82" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C7" s="83" t="s">
-        <v>81</v>
-      </c>
-      <c r="D7" s="83" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="82" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C8" s="83" t="s">
-        <v>83</v>
-      </c>
-      <c r="D8" s="83" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="82" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C9" s="83" t="s">
-        <v>86</v>
-      </c>
-      <c r="D9" s="83" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -7042,7 +6983,7 @@
   <sheetData>
     <row r="2" s="2" customFormat="true" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="84" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7059,7 +7000,7 @@
       <c r="L4" s="15"/>
       <c r="M4" s="15"/>
       <c r="N4" s="85" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="O4" s="85"/>
       <c r="P4" s="85"/>
@@ -7067,14 +7008,14 @@
       <c r="R4" s="85"/>
       <c r="S4" s="15"/>
       <c r="T4" s="85" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="U4" s="85"/>
       <c r="V4" s="85"/>
       <c r="W4" s="85"/>
       <c r="X4" s="85"/>
       <c r="Y4" s="86" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="Z4" s="86"/>
     </row>
@@ -7086,49 +7027,49 @@
       <c r="F5" s="33"/>
       <c r="G5" s="33"/>
       <c r="H5" s="87" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="I5" s="88"/>
       <c r="J5" s="87" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="K5" s="88"/>
       <c r="L5" s="87" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="M5" s="89"/>
       <c r="N5" s="87" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="O5" s="87" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="P5" s="88"/>
       <c r="Q5" s="87" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="R5" s="87" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="S5" s="88"/>
       <c r="T5" s="87" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="U5" s="87" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="V5" s="88"/>
       <c r="W5" s="87" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="X5" s="87" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="Y5" s="87" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="Z5" s="87" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7137,68 +7078,68 @@
       </c>
       <c r="C6" s="88"/>
       <c r="D6" s="91" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="E6" s="91"/>
       <c r="F6" s="91"/>
       <c r="G6" s="88"/>
       <c r="H6" s="90" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="I6" s="88"/>
       <c r="J6" s="90" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="K6" s="88"/>
       <c r="L6" s="90" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="M6" s="15"/>
       <c r="N6" s="90" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="O6" s="90" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="P6" s="88"/>
       <c r="Q6" s="90" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="R6" s="90" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="S6" s="15"/>
       <c r="T6" s="90" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="U6" s="90" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="V6" s="90" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="W6" s="90" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="X6" s="90" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Y6" s="90" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Z6" s="90" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="H7" s="92" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="J7" s="92" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="L7" s="92" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7207,7 +7148,7 @@
       </c>
       <c r="C8" s="94"/>
       <c r="D8" s="95" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="E8" s="95"/>
       <c r="F8" s="95"/>
@@ -7298,11 +7239,11 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="107" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C10" s="102"/>
       <c r="D10" s="108" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="E10" s="108"/>
       <c r="F10" s="108"/>
@@ -7355,11 +7296,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="107" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="C11" s="102"/>
       <c r="D11" s="108" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="E11" s="108"/>
       <c r="F11" s="108"/>
@@ -7412,11 +7353,11 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="107" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C12" s="102"/>
       <c r="D12" s="108" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="E12" s="108"/>
       <c r="F12" s="108"/>
@@ -7469,11 +7410,11 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="107" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C13" s="102"/>
       <c r="D13" s="108" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="E13" s="108"/>
       <c r="F13" s="108"/>
@@ -7526,11 +7467,11 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="107" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="C14" s="102"/>
       <c r="D14" s="108" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="E14" s="108"/>
       <c r="F14" s="108"/>
@@ -7689,7 +7630,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="117" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="C20" s="118"/>
       <c r="D20" s="118"/>
@@ -7757,7 +7698,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="117" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="C21" s="118"/>
       <c r="D21" s="118"/>
@@ -7825,7 +7766,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="123" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="C24" s="61"/>
       <c r="D24" s="61"/>
@@ -7838,36 +7779,36 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="87" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="C25" s="87" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D25" s="87" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="E25" s="87" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="F25" s="87" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G25" s="87" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="H25" s="87" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="I25" s="87" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="J25" s="87" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="124" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="C26" s="125" t="n">
         <f aca="false">U21</f>
@@ -7904,7 +7845,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="129" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="C27" s="130" t="n">
         <f aca="false">X21</f>
@@ -7941,7 +7882,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="124" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="C28" s="125" t="n">
         <f aca="false">Z21</f>
@@ -7978,7 +7919,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="134" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -8020,17 +7961,17 @@
   <sheetData>
     <row r="2" s="2" customFormat="true" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="8" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="8" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8038,10 +7979,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="123" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B7" s="74" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C7" s="33"/>
       <c r="D7" s="33"/>
@@ -8050,7 +7991,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="F8" s="54" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$8*'Sources &amp; Checks'!$B$5</f>
@@ -8059,7 +8000,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="8" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="F9" s="27" t="n">
         <f aca="false">F8/(F8+F15)</f>
@@ -8068,7 +8009,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="F10" s="136" t="n">
         <f aca="false">F11+F14*F13</f>
@@ -8077,7 +8018,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="F11" s="37" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$10</f>
@@ -8086,7 +8027,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="8" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="F12" s="137" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$11</f>
@@ -8095,7 +8036,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="8" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="F13" s="37" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$12</f>
@@ -8104,7 +8045,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="F14" s="138" t="n">
         <f aca="false">1/3*1+2/3*F12</f>
@@ -8113,10 +8054,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="123" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B15" s="74" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="F15" s="139" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$7</f>
@@ -8125,7 +8066,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="8" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="F16" s="38" t="n">
         <f aca="false">F15/(F15+F8)</f>
@@ -8134,7 +8075,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="8" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F17" s="38" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$13</f>
@@ -8143,7 +8084,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="F18" s="38" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$14</f>
@@ -8152,10 +8093,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="123" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B20" s="74" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="F20" s="54" t="n">
         <f aca="false">F15+F8</f>
@@ -8164,10 +8105,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="123" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B22" s="74" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F22" s="140" t="n">
         <f aca="false">F9*F10+(F16*F17*(1-F18))</f>
@@ -8202,7 +8143,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="141" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="B1" s="141"/>
       <c r="C1" s="141"/>
@@ -8210,270 +8151,270 @@
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="87" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="B3" s="87" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="C3" s="87" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="D3" s="87" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="142" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="B4" s="143" t="n">
         <v>46087</v>
       </c>
       <c r="C4" s="142" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="D4" s="142" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="142" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="B5" s="144" t="n">
         <v>26.19</v>
       </c>
       <c r="C5" s="142" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="D5" s="142" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="142" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="B6" s="145" t="n">
         <v>2400</v>
       </c>
       <c r="C6" s="142" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="D6" s="142" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="142" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="B7" s="145" t="n">
         <v>1500</v>
       </c>
       <c r="C7" s="142" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="D7" s="142" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="142" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="B8" s="145" t="n">
         <v>1050</v>
       </c>
       <c r="C8" s="142" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="D8" s="142" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="142" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="B9" s="145" t="n">
         <v>1066.8</v>
       </c>
       <c r="C9" s="142" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="D9" s="142" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="142" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="B10" s="146" t="n">
         <v>0.028643</v>
       </c>
       <c r="C10" s="142" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D10" s="142" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="142" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="B11" s="147" t="n">
         <v>1.01</v>
       </c>
       <c r="C11" s="142" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="D11" s="142" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="142" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="B12" s="146" t="n">
         <v>0.06</v>
       </c>
       <c r="C12" s="142" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D12" s="142" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="142" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="B13" s="146" t="n">
         <v>0.03</v>
       </c>
       <c r="C13" s="142" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D13" s="142" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="142" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B14" s="146" t="n">
         <v>0.12</v>
       </c>
       <c r="C14" s="142" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D14" s="142" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="148" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="B16" s="148" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="148" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="B18" s="148" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="C18" s="148" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="D18" s="148" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="148" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="B19" s="149" t="n">
         <v>0.0909</v>
       </c>
       <c r="C19" s="148" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D19" s="148" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="148" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="B20" s="149" t="n">
         <v>0.1722</v>
       </c>
       <c r="C20" s="148" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D20" s="148" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="148" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="B21" s="149" t="n">
         <v>0.0805</v>
       </c>
       <c r="C21" s="148" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D21" s="148" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="148" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="B22" s="149" t="n">
         <v>0.1828</v>
       </c>
       <c r="C22" s="148" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D22" s="148" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="148" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="B23" s="149" t="n">
         <v>-0.0287</v>
       </c>
       <c r="C23" s="148" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D23" s="148" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="150" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="B25" s="151" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -8511,21 +8452,21 @@
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="154" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C3" s="155" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="D3" s="156" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="E3" s="157" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="158" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="C4" s="159" t="n">
         <v>10775</v>
@@ -8539,7 +8480,7 @@
     </row>
     <row r="5" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="162" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="C5" s="163" t="n">
         <v>9332</v>
@@ -8553,7 +8494,7 @@
     </row>
     <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="162" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="C6" s="163" t="n">
         <v>1443</v>
@@ -8567,7 +8508,7 @@
     </row>
     <row r="7" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="166" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="C7" s="167" t="n">
         <v>1314</v>
@@ -8581,21 +8522,21 @@
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="154" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="C10" s="155" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="D10" s="156" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="E10" s="157" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="158" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="C11" s="159" t="n">
         <v>16406</v>
@@ -8609,7 +8550,7 @@
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="162" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C12" s="163" t="n">
         <v>5643</v>
@@ -8623,7 +8564,7 @@
     </row>
     <row r="13" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="166" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="C13" s="167" t="n">
         <v>4675</v>
@@ -8637,21 +8578,21 @@
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="154" t="s">
-        <v>146</v>
+        <v>202</v>
       </c>
       <c r="C16" s="155" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="D16" s="156" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="E16" s="157" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="158" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="C17" s="159" t="n">
         <v>7422</v>
@@ -8665,7 +8606,7 @@
     </row>
     <row r="18" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="162" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="C18" s="163" t="n">
         <v>3341</v>
@@ -8679,7 +8620,7 @@
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="170" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="C19" s="171" t="n">
         <f aca="false">C17+C18</f>
@@ -8696,21 +8637,21 @@
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="154" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="C22" s="155" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="D22" s="156" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="E22" s="157" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="158" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="C23" s="174" t="n">
         <f aca="false">(C4-4800.9)/4800.9</f>
@@ -8727,10 +8668,10 @@
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="162" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="C24" s="176" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="D24" s="177" t="n">
         <f aca="false">(D7-C7)/C7</f>
@@ -8743,7 +8684,7 @@
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="162" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="C25" s="179" t="n">
         <f aca="false">C7/C4</f>
@@ -8760,7 +8701,7 @@
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="162" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="C26" s="179" t="n">
         <f aca="false">(C4-C5)/C4</f>
@@ -8777,7 +8718,7 @@
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="162" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="C27" s="179" t="n">
         <f aca="false">C5/C4</f>
@@ -8794,7 +8735,7 @@
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="162" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="C28" s="179" t="n">
         <f aca="false">C7/C11</f>
@@ -8811,7 +8752,7 @@
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="162" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="C29" s="179" t="n">
         <f aca="false">C7/C12</f>
@@ -8828,7 +8769,7 @@
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="162" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="C30" s="179" t="n">
         <f aca="false">C19/C11</f>
@@ -8845,7 +8786,7 @@
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="166" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="C31" s="180" t="n">
         <f aca="false">C12/C11</f>
@@ -8862,17 +8803,17 @@
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="152" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="152" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="152" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -8904,18 +8845,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="80" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="81" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="C3" s="81"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="83" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C4" s="183" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$14</f>
@@ -8924,7 +8865,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="83" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="C5" s="184" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$21</f>
@@ -8933,7 +8874,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="83" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="C6" s="184" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$22</f>
@@ -8942,7 +8883,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="83" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="C7" s="184" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$23</f>
@@ -8951,7 +8892,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="83" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="C8" s="185" t="n">
         <f aca="false">DCF!$N$20</f>
@@ -8960,7 +8901,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="83" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="C9" s="185" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$6</f>
@@ -8969,7 +8910,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="83" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="C10" s="185" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$7</f>
@@ -8978,7 +8919,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="83" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="C11" s="185" t="n">
         <f aca="false">'Sources &amp; Checks'!$B$9</f>
@@ -8987,7 +8928,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="83" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C12" s="186" t="n">
         <f aca="false">DCF!$D$18</f>
@@ -8996,12 +8937,12 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="187" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="81" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C15" s="81"/>
       <c r="D15" s="81"/>
@@ -9020,13 +8961,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="188" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="C16" s="188" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="E16" s="188" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="F16" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -9069,19 +9010,19 @@
         <v>FY35</v>
       </c>
       <c r="P16" s="189" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="83" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C17" s="184" t="n">
         <f aca="false">DCF!$H$11</f>
         <v>0.07</v>
       </c>
       <c r="E17" s="83" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F17" s="190" t="n">
         <f aca="false">$C$17</f>
@@ -9126,14 +9067,14 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="83" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C18" s="184" t="n">
         <f aca="false">DCF!$H$13</f>
         <v>0.16</v>
       </c>
       <c r="E18" s="83" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F18" s="191" t="n">
         <f aca="false">$C$8*(1+F17)</f>
@@ -9178,14 +9119,14 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="83" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C19" s="192" t="n">
         <f aca="false">DCF!$H$16</f>
         <v>0.092</v>
       </c>
       <c r="E19" s="83" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="F19" s="191" t="n">
         <f aca="false">F18*$C$18*(1-$C$4)</f>
@@ -9234,14 +9175,14 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="83" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="C20" s="184" t="n">
         <f aca="false">DCF!$H$17</f>
         <v>0.01</v>
       </c>
       <c r="E20" s="83" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F20" s="190" t="n">
         <f aca="false">$C$17/(($C$6-$C$5+$C$7)/($C$18*(1-$C$4)))</f>
@@ -9290,7 +9231,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E21" s="83" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F21" s="193" t="n">
         <f aca="false">F17/F20</f>
@@ -9339,7 +9280,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E22" s="83" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="F22" s="191" t="n">
         <f aca="false">F19*F21</f>
@@ -9384,7 +9325,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E23" s="82" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F23" s="194" t="n">
         <f aca="false">F19-F22</f>
@@ -9433,14 +9374,14 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="83" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="C24" s="185" t="n">
         <f aca="false">SUM(F25:O25)</f>
         <v>10677.2345379775</v>
       </c>
       <c r="E24" s="83" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="F24" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -9485,14 +9426,14 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="83" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C25" s="185" t="n">
         <f aca="false">P23/($C$19-$C$20)</f>
         <v>31861.0982339967</v>
       </c>
       <c r="E25" s="83" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="F25" s="191" t="n">
         <f aca="false">F23*DCF!$O$70/(1+$C$19)^F24</f>
@@ -9537,7 +9478,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="83" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="C26" s="185" t="n">
         <f aca="false">C25/(1+$C$19)^O24</f>
@@ -9546,7 +9487,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="83" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="C27" s="185" t="n">
         <f aca="false">C24+C26</f>
@@ -9555,7 +9496,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="83" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C28" s="185" t="n">
         <f aca="false">C27+$C$9-$C$10</f>
@@ -9564,7 +9505,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="188" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C29" s="196" t="n">
         <f aca="false">C28/$C$11</f>
@@ -9573,7 +9514,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="83" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="C30" s="183" t="n">
         <f aca="false">1-P23/P19</f>
@@ -9582,7 +9523,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="83" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C31" s="183" t="n">
         <f aca="false">C26/C27</f>
@@ -9591,7 +9532,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="81" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C34" s="81"/>
       <c r="D34" s="81"/>
@@ -9610,13 +9551,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="188" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="C35" s="188" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="E35" s="188" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="F35" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -9659,19 +9600,19 @@
         <v>FY35</v>
       </c>
       <c r="P35" s="189" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="83" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C36" s="184" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E36" s="83" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F36" s="190" t="n">
         <f aca="false">$C$36</f>
@@ -9716,14 +9657,14 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="83" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C37" s="184" t="n">
         <f aca="false">DCF!$L$13</f>
         <v>0.1722</v>
       </c>
       <c r="E37" s="83" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F37" s="191" t="n">
         <f aca="false">$C$8*(1+F36)</f>
@@ -9768,14 +9709,14 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="83" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C38" s="192" t="n">
         <f aca="false">DCF!$L$16</f>
         <v>0.0858027889618787</v>
       </c>
       <c r="E38" s="83" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="F38" s="191" t="n">
         <f aca="false">F37*$C$37*(1-$C$4)</f>
@@ -9824,14 +9765,14 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="83" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="C39" s="184" t="n">
         <f aca="false">DCF!$L$17</f>
         <v>0.015</v>
       </c>
       <c r="E39" s="83" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F39" s="190" t="n">
         <f aca="false">$C$36/(($C$6-$C$5+$C$7)/($C$37*(1-$C$4)))</f>
@@ -9880,7 +9821,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E40" s="83" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F40" s="193" t="n">
         <f aca="false">F36/F39</f>
@@ -9929,7 +9870,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E41" s="83" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="F41" s="191" t="n">
         <f aca="false">F38*F40</f>
@@ -9974,7 +9915,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E42" s="82" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F42" s="194" t="n">
         <f aca="false">F38-F41</f>
@@ -10023,14 +9964,14 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="83" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="C43" s="185" t="n">
         <f aca="false">SUM(F44:O44)</f>
         <v>12309.8454096608</v>
       </c>
       <c r="E43" s="83" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="F43" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -10075,14 +10016,14 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="83" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C44" s="185" t="n">
         <f aca="false">P42/($C$38-$C$39)</f>
         <v>41776.8531981022</v>
       </c>
       <c r="E44" s="83" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="F44" s="191" t="n">
         <f aca="false">F42*DCF!$O$70/(1+$C$38)^F43</f>
@@ -10127,7 +10068,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="83" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="C45" s="185" t="n">
         <f aca="false">C44/(1+$C$38)^O43</f>
@@ -10136,7 +10077,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="83" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="C46" s="185" t="n">
         <f aca="false">C43+C45</f>
@@ -10145,7 +10086,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="83" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C47" s="185" t="n">
         <f aca="false">C46+$C$9-$C$10</f>
@@ -10154,7 +10095,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="188" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C48" s="196" t="n">
         <f aca="false">C47/$C$11</f>
@@ -10163,7 +10104,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="83" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="C49" s="183" t="n">
         <f aca="false">1-P42/P38</f>
@@ -10172,7 +10113,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="83" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C50" s="183" t="n">
         <f aca="false">C45/C46</f>
@@ -10181,7 +10122,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="81" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C53" s="81"/>
       <c r="D53" s="81"/>
@@ -10200,13 +10141,13 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="188" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="C54" s="188" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="E54" s="188" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="F54" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -10249,19 +10190,19 @@
         <v>FY35</v>
       </c>
       <c r="P54" s="189" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="83" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C55" s="184" t="n">
         <f aca="false">DCF!$P$11</f>
         <v>0.11</v>
       </c>
       <c r="E55" s="83" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F55" s="190" t="n">
         <f aca="false">$C$55</f>
@@ -10306,14 +10247,14 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="83" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C56" s="184" t="n">
         <f aca="false">DCF!$P$13</f>
         <v>0.185</v>
       </c>
       <c r="E56" s="83" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F56" s="191" t="n">
         <f aca="false">$C$8*(1+F55)</f>
@@ -10358,14 +10299,14 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="83" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C57" s="192" t="n">
         <f aca="false">DCF!$P$16</f>
         <v>0.082</v>
       </c>
       <c r="E57" s="83" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="F57" s="191" t="n">
         <f aca="false">F56*$C$56*(1-$C$4)</f>
@@ -10414,14 +10355,14 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="83" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="C58" s="184" t="n">
         <f aca="false">DCF!$P$17</f>
         <v>0.02</v>
       </c>
       <c r="E58" s="83" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F58" s="190" t="n">
         <f aca="false">$C$55/(($C$6-$C$5+$C$7)/($C$56*(1-$C$4)))</f>
@@ -10470,7 +10411,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E59" s="83" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F59" s="193" t="n">
         <f aca="false">F55/F58</f>
@@ -10519,7 +10460,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E60" s="83" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="F60" s="191" t="n">
         <f aca="false">F57*F59</f>
@@ -10564,7 +10505,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E61" s="82" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F61" s="194" t="n">
         <f aca="false">F57-F60</f>
@@ -10613,14 +10554,14 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B62" s="83" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="C62" s="185" t="n">
         <f aca="false">SUM(F63:O63)</f>
         <v>14171.7844838877</v>
       </c>
       <c r="E62" s="83" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="F62" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -10665,14 +10606,14 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B63" s="83" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C63" s="185" t="n">
         <f aca="false">P61/($C$57-$C$58)</f>
         <v>52830.3906260597</v>
       </c>
       <c r="E63" s="83" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="F63" s="191" t="n">
         <f aca="false">F61*DCF!$O$70/(1+$C$57)^F62</f>
@@ -10717,7 +10658,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="83" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="C64" s="185" t="n">
         <f aca="false">C63/(1+$C$57)^O62</f>
@@ -10726,7 +10667,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="83" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="C65" s="185" t="n">
         <f aca="false">C62+C64</f>
@@ -10735,7 +10676,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B66" s="83" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C66" s="185" t="n">
         <f aca="false">C65+$C$9-$C$10</f>
@@ -10744,7 +10685,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B67" s="188" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C67" s="196" t="n">
         <f aca="false">C66/$C$11</f>
@@ -10753,7 +10694,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B68" s="83" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="C68" s="183" t="n">
         <f aca="false">1-P61/P57</f>
@@ -10762,7 +10703,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B69" s="83" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C69" s="183" t="n">
         <f aca="false">C64/C65</f>
@@ -10771,12 +10712,13 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B72" s="187" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B73" s="81" t="s">
-        <v>254</v>
+      <c r="B73" s="81" t="str">
+        <f aca="false">"Sensitivity, terminal growth "&amp;TEXT(DCF!$D$92,"0.0%")</f>
+        <v>Sensitivity, terminal growth 0.5%</v>
       </c>
       <c r="C73" s="81"/>
       <c r="D73" s="81"/>
@@ -10795,13 +10737,13 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B74" s="188" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="C74" s="188" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="E74" s="188" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="F74" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -10844,19 +10786,19 @@
         <v>FY35</v>
       </c>
       <c r="P74" s="189" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B75" s="83" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C75" s="184" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E75" s="83" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F75" s="190" t="n">
         <f aca="false">$C$75</f>
@@ -10901,14 +10843,14 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B76" s="83" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C76" s="184" t="n">
         <f aca="false">DCF!$L$13</f>
         <v>0.1722</v>
       </c>
       <c r="E76" s="83" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F76" s="191" t="n">
         <f aca="false">$C$8*(1+F75)</f>
@@ -10953,14 +10895,14 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B77" s="83" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C77" s="192" t="n">
         <f aca="false">DCF!$L$16</f>
         <v>0.0858027889618787</v>
       </c>
       <c r="E77" s="83" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="F77" s="191" t="n">
         <f aca="false">F76*$C$76*(1-$C$4)</f>
@@ -11009,14 +10951,14 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B78" s="83" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="C78" s="184" t="n">
         <f aca="false">DCF!$D$92</f>
         <v>0.005</v>
       </c>
       <c r="E78" s="83" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F78" s="190" t="n">
         <f aca="false">$C$75/(($C$6-$C$5+$C$7)/($C$76*(1-$C$4)))</f>
@@ -11065,7 +11007,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E79" s="83" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F79" s="193" t="n">
         <f aca="false">F75/F78</f>
@@ -11114,7 +11056,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E80" s="83" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="F80" s="191" t="n">
         <f aca="false">F77*F79</f>
@@ -11159,7 +11101,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E81" s="82" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F81" s="194" t="n">
         <f aca="false">F77-F80</f>
@@ -11208,14 +11150,14 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B82" s="83" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="C82" s="185" t="n">
         <f aca="false">SUM(F83:O83)</f>
         <v>12935.2230595844</v>
       </c>
       <c r="E82" s="83" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="F82" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -11260,14 +11202,14 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B83" s="83" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C83" s="185" t="n">
         <f aca="false">P81/($C$77-$C$78)</f>
         <v>39411.8359558047</v>
       </c>
       <c r="E83" s="83" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="F83" s="191" t="n">
         <f aca="false">F81*DCF!$O$70/(1+$C$77)^F82</f>
@@ -11312,7 +11254,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B84" s="83" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="C84" s="185" t="n">
         <f aca="false">C83/(1+$C$77)^O82</f>
@@ -11321,7 +11263,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B85" s="83" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="C85" s="185" t="n">
         <f aca="false">C82+C84</f>
@@ -11330,7 +11272,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B86" s="83" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C86" s="185" t="n">
         <f aca="false">C85+$C$9-$C$10</f>
@@ -11339,7 +11281,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B87" s="188" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C87" s="196" t="n">
         <f aca="false">C86/$C$11</f>
@@ -11348,7 +11290,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B88" s="83" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="C88" s="183" t="n">
         <f aca="false">1-P81/P77</f>
@@ -11357,7 +11299,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B89" s="83" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C89" s="183" t="n">
         <f aca="false">C84/C85</f>
@@ -11365,8 +11307,9 @@
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B92" s="81" t="s">
-        <v>255</v>
+      <c r="B92" s="81" t="str">
+        <f aca="false">"Sensitivity, terminal growth "&amp;TEXT(DCF!$F$92,"0.0%")</f>
+        <v>Sensitivity, terminal growth 1.0%</v>
       </c>
       <c r="C92" s="81"/>
       <c r="D92" s="81"/>
@@ -11385,13 +11328,13 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B93" s="188" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="C93" s="188" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="E93" s="188" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="F93" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -11434,19 +11377,19 @@
         <v>FY35</v>
       </c>
       <c r="P93" s="189" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B94" s="83" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C94" s="184" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E94" s="83" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F94" s="190" t="n">
         <f aca="false">$C$94</f>
@@ -11491,14 +11434,14 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B95" s="83" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C95" s="184" t="n">
         <f aca="false">DCF!$L$13</f>
         <v>0.1722</v>
       </c>
       <c r="E95" s="83" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F95" s="191" t="n">
         <f aca="false">$C$8*(1+F94)</f>
@@ -11543,14 +11486,14 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B96" s="83" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C96" s="192" t="n">
         <f aca="false">DCF!$L$16</f>
         <v>0.0858027889618787</v>
       </c>
       <c r="E96" s="83" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="F96" s="191" t="n">
         <f aca="false">F95*$C$95*(1-$C$4)</f>
@@ -11599,14 +11542,14 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B97" s="83" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="C97" s="184" t="n">
         <f aca="false">DCF!$F$92</f>
         <v>0.01</v>
       </c>
       <c r="E97" s="83" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F97" s="190" t="n">
         <f aca="false">$C$94/(($C$6-$C$5+$C$7)/($C$95*(1-$C$4)))</f>
@@ -11655,7 +11598,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E98" s="83" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F98" s="193" t="n">
         <f aca="false">F94/F97</f>
@@ -11704,7 +11647,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E99" s="83" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="F99" s="191" t="n">
         <f aca="false">F96*F98</f>
@@ -11749,7 +11692,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E100" s="82" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F100" s="194" t="n">
         <f aca="false">F96-F99</f>
@@ -11798,14 +11741,14 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B101" s="83" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="C101" s="185" t="n">
         <f aca="false">SUM(F102:O102)</f>
         <v>12628.0179564231</v>
       </c>
       <c r="E101" s="83" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="F101" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -11850,14 +11793,14 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B102" s="83" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C102" s="185" t="n">
         <f aca="false">P100/($C$96-$C$97)</f>
         <v>40579.3082501446</v>
       </c>
       <c r="E102" s="83" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="F102" s="191" t="n">
         <f aca="false">F100*DCF!$O$70/(1+$C$96)^F101</f>
@@ -11902,7 +11845,7 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B103" s="83" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="C103" s="185" t="n">
         <f aca="false">C102/(1+$C$96)^O101</f>
@@ -11911,7 +11854,7 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B104" s="83" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="C104" s="185" t="n">
         <f aca="false">C101+C103</f>
@@ -11920,7 +11863,7 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B105" s="83" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C105" s="185" t="n">
         <f aca="false">C104+$C$9-$C$10</f>
@@ -11929,7 +11872,7 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B106" s="188" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C106" s="196" t="n">
         <f aca="false">C105/$C$11</f>
@@ -11938,7 +11881,7 @@
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B107" s="83" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="C107" s="183" t="n">
         <f aca="false">1-P100/P96</f>
@@ -11947,7 +11890,7 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B108" s="83" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C108" s="183" t="n">
         <f aca="false">C103/C104</f>
@@ -11955,8 +11898,9 @@
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B111" s="81" t="s">
-        <v>256</v>
+      <c r="B111" s="81" t="str">
+        <f aca="false">"Sensitivity, terminal growth "&amp;TEXT(DCF!$H$92,"0.0%")</f>
+        <v>Sensitivity, terminal growth 1.5%</v>
       </c>
       <c r="C111" s="81"/>
       <c r="D111" s="81"/>
@@ -11975,13 +11919,13 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B112" s="188" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="C112" s="188" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="E112" s="188" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="F112" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -12024,19 +11968,19 @@
         <v>FY35</v>
       </c>
       <c r="P112" s="189" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B113" s="83" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C113" s="184" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E113" s="83" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F113" s="190" t="n">
         <f aca="false">$C$113</f>
@@ -12081,14 +12025,14 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B114" s="83" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C114" s="184" t="n">
         <f aca="false">DCF!$L$13</f>
         <v>0.1722</v>
       </c>
       <c r="E114" s="83" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F114" s="191" t="n">
         <f aca="false">$C$8*(1+F113)</f>
@@ -12133,14 +12077,14 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B115" s="83" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C115" s="192" t="n">
         <f aca="false">DCF!$L$16</f>
         <v>0.0858027889618787</v>
       </c>
       <c r="E115" s="83" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="F115" s="191" t="n">
         <f aca="false">F114*$C$114*(1-$C$4)</f>
@@ -12189,14 +12133,14 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B116" s="83" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="C116" s="184" t="n">
         <f aca="false">DCF!$H$92</f>
         <v>0.015</v>
       </c>
       <c r="E116" s="83" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F116" s="190" t="n">
         <f aca="false">$C$113/(($C$6-$C$5+$C$7)/($C$114*(1-$C$4)))</f>
@@ -12245,7 +12189,7 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E117" s="83" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F117" s="193" t="n">
         <f aca="false">F113/F116</f>
@@ -12294,7 +12238,7 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E118" s="83" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="F118" s="191" t="n">
         <f aca="false">F115*F117</f>
@@ -12339,7 +12283,7 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E119" s="82" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F119" s="194" t="n">
         <f aca="false">F115-F118</f>
@@ -12388,14 +12332,14 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B120" s="83" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="C120" s="185" t="n">
         <f aca="false">SUM(F121:O121)</f>
         <v>12309.8454096608</v>
       </c>
       <c r="E120" s="83" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="F120" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -12440,14 +12384,14 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B121" s="83" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C121" s="185" t="n">
         <f aca="false">P119/($C$115-$C$116)</f>
         <v>41776.8531981022</v>
       </c>
       <c r="E121" s="83" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="F121" s="191" t="n">
         <f aca="false">F119*DCF!$O$70/(1+$C$115)^F120</f>
@@ -12492,7 +12436,7 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B122" s="83" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="C122" s="185" t="n">
         <f aca="false">C121/(1+$C$115)^O120</f>
@@ -12501,7 +12445,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B123" s="83" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="C123" s="185" t="n">
         <f aca="false">C120+C122</f>
@@ -12510,7 +12454,7 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B124" s="83" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C124" s="185" t="n">
         <f aca="false">C123+$C$9-$C$10</f>
@@ -12519,7 +12463,7 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B125" s="188" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C125" s="196" t="n">
         <f aca="false">C124/$C$11</f>
@@ -12528,7 +12472,7 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B126" s="83" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="C126" s="183" t="n">
         <f aca="false">1-P119/P115</f>
@@ -12537,7 +12481,7 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B127" s="83" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C127" s="183" t="n">
         <f aca="false">C122/C123</f>
@@ -12545,8 +12489,9 @@
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B130" s="81" t="s">
-        <v>257</v>
+      <c r="B130" s="81" t="str">
+        <f aca="false">"Sensitivity, terminal growth "&amp;TEXT(DCF!$J$92,"0.0%")</f>
+        <v>Sensitivity, terminal growth 2.0%</v>
       </c>
       <c r="C130" s="81"/>
       <c r="D130" s="81"/>
@@ -12565,13 +12510,13 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B131" s="188" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="C131" s="188" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="E131" s="188" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="F131" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -12614,19 +12559,19 @@
         <v>FY35</v>
       </c>
       <c r="P131" s="189" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B132" s="83" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C132" s="184" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E132" s="83" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F132" s="190" t="n">
         <f aca="false">$C$132</f>
@@ -12671,14 +12616,14 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B133" s="83" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C133" s="184" t="n">
         <f aca="false">DCF!$L$13</f>
         <v>0.1722</v>
       </c>
       <c r="E133" s="83" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F133" s="191" t="n">
         <f aca="false">$C$8*(1+F132)</f>
@@ -12723,14 +12668,14 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B134" s="83" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C134" s="192" t="n">
         <f aca="false">DCF!$L$16</f>
         <v>0.0858027889618787</v>
       </c>
       <c r="E134" s="83" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="F134" s="191" t="n">
         <f aca="false">F133*$C$133*(1-$C$4)</f>
@@ -12779,14 +12724,14 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B135" s="83" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="C135" s="184" t="n">
         <f aca="false">DCF!$J$92</f>
         <v>0.02</v>
       </c>
       <c r="E135" s="83" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F135" s="190" t="n">
         <f aca="false">$C$132/(($C$6-$C$5+$C$7)/($C$133*(1-$C$4)))</f>
@@ -12835,7 +12780,7 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E136" s="83" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F136" s="193" t="n">
         <f aca="false">F132/F135</f>
@@ -12884,7 +12829,7 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E137" s="83" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="F137" s="191" t="n">
         <f aca="false">F134*F136</f>
@@ -12929,7 +12874,7 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E138" s="82" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F138" s="194" t="n">
         <f aca="false">F134-F137</f>
@@ -12978,14 +12923,14 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B139" s="83" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="C139" s="185" t="n">
         <f aca="false">SUM(F140:O140)</f>
         <v>11980.4344599675</v>
       </c>
       <c r="E139" s="83" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="F139" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -13030,14 +12975,14 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B140" s="83" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C140" s="185" t="n">
         <f aca="false">P138/($C$134-$C$135)</f>
         <v>43005.1340184788</v>
       </c>
       <c r="E140" s="83" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="F140" s="191" t="n">
         <f aca="false">F138*DCF!$O$70/(1+$C$134)^F139</f>
@@ -13082,7 +13027,7 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B141" s="83" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="C141" s="185" t="n">
         <f aca="false">C140/(1+$C$134)^O139</f>
@@ -13091,7 +13036,7 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B142" s="83" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="C142" s="185" t="n">
         <f aca="false">C139+C141</f>
@@ -13100,7 +13045,7 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B143" s="83" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C143" s="185" t="n">
         <f aca="false">C142+$C$9-$C$10</f>
@@ -13109,7 +13054,7 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B144" s="188" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C144" s="196" t="n">
         <f aca="false">C143/$C$11</f>
@@ -13118,7 +13063,7 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B145" s="83" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="C145" s="183" t="n">
         <f aca="false">1-P138/P134</f>
@@ -13127,7 +13072,7 @@
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B146" s="83" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C146" s="183" t="n">
         <f aca="false">C141/C142</f>
@@ -13135,8 +13080,9 @@
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B149" s="81" t="s">
-        <v>258</v>
+      <c r="B149" s="81" t="str">
+        <f aca="false">"Sensitivity, terminal growth "&amp;TEXT(DCF!$L$92,"0.0%")</f>
+        <v>Sensitivity, terminal growth 2.5%</v>
       </c>
       <c r="C149" s="81"/>
       <c r="D149" s="81"/>
@@ -13155,13 +13101,13 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B150" s="188" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="C150" s="188" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="E150" s="188" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="F150" s="189" t="str">
         <f aca="false">"FY"&amp;RIGHT(DCF!O$38,2)</f>
@@ -13204,19 +13150,19 @@
         <v>FY35</v>
       </c>
       <c r="P150" s="189" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B151" s="83" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C151" s="184" t="n">
         <f aca="false">DCF!$L$11</f>
         <v>0.0909</v>
       </c>
       <c r="E151" s="83" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F151" s="190" t="n">
         <f aca="false">$C$151</f>
@@ -13261,14 +13207,14 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B152" s="83" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C152" s="184" t="n">
         <f aca="false">DCF!$L$13</f>
         <v>0.1722</v>
       </c>
       <c r="E152" s="83" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F152" s="191" t="n">
         <f aca="false">$C$8*(1+F151)</f>
@@ -13313,14 +13259,14 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B153" s="83" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C153" s="192" t="n">
         <f aca="false">DCF!$L$16</f>
         <v>0.0858027889618787</v>
       </c>
       <c r="E153" s="83" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="F153" s="191" t="n">
         <f aca="false">F152*$C$152*(1-$C$4)</f>
@@ -13369,14 +13315,14 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B154" s="83" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="C154" s="184" t="n">
         <f aca="false">DCF!$L$92</f>
         <v>0.025</v>
       </c>
       <c r="E154" s="83" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F154" s="190" t="n">
         <f aca="false">$C$151/(($C$6-$C$5+$C$7)/($C$152*(1-$C$4)))</f>
@@ -13425,7 +13371,7 @@
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E155" s="83" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F155" s="193" t="n">
         <f aca="false">F151/F154</f>
@@ -13474,7 +13420,7 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E156" s="83" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="F156" s="191" t="n">
         <f aca="false">F153*F155</f>
@@ -13519,7 +13465,7 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E157" s="82" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F157" s="194" t="n">
         <f aca="false">F153-F156</f>
@@ -13568,14 +13514,14 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B158" s="83" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="C158" s="185" t="n">
         <f aca="false">SUM(F159:O159)</f>
         <v>11639.5088061378</v>
       </c>
       <c r="E158" s="83" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="F158" s="195" t="n">
         <f aca="false">DCF!O$71</f>
@@ -13620,14 +13566,14 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B159" s="83" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C159" s="185" t="n">
         <f aca="false">P157/($C$153-$C$154)</f>
         <v>44264.8262118657</v>
       </c>
       <c r="E159" s="83" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="F159" s="191" t="n">
         <f aca="false">F157*DCF!$O$70/(1+$C$153)^F158</f>
@@ -13672,7 +13618,7 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B160" s="83" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="C160" s="185" t="n">
         <f aca="false">C159/(1+$C$153)^O158</f>
@@ -13681,7 +13627,7 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B161" s="83" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="C161" s="185" t="n">
         <f aca="false">C158+C160</f>
@@ -13690,7 +13636,7 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B162" s="83" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C162" s="185" t="n">
         <f aca="false">C161+$C$9-$C$10</f>
@@ -13699,7 +13645,7 @@
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B163" s="188" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C163" s="196" t="n">
         <f aca="false">C162/$C$11</f>
@@ -13708,7 +13654,7 @@
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B164" s="83" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="C164" s="183" t="n">
         <f aca="false">1-P157/P153</f>
@@ -13717,7 +13663,7 @@
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B165" s="83" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C165" s="183" t="n">
         <f aca="false">C160/C161</f>

</xml_diff>

<commit_message>
Use plain text for note cells
</commit_message>
<xml_diff>
--- a/Ryanair_DCF_Model_Kodickova_2026.xlsx
+++ b/Ryanair_DCF_Model_Kodickova_2026.xlsx
@@ -6861,9 +6861,10 @@
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B101" s="79" t="str">
-        <f aca="false">"⬛ = base case (WACC "&amp;ROUND(WACC!$F$22*100,2)&amp;"%"&amp;", TGR "&amp;ROUND(DCF!$L$17*100,1)&amp;"%"&amp;"). Each TGR column uses its own growth path, fading to that rate by FY35. The WACC rows change discounting and terminal value only. Current price: €"&amp;ROUND('Sources &amp; Checks'!$B$5,2)&amp;"."</f>
-        <v>⬛ = base case (WACC 8.58%, TGR 1.5%). Each TGR column uses its own growth path, fading to that rate by FY35. The WACC rows change discounting and terminal value only. Current price: €26.19.</v>
+      <c r="B101" s="79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⬛ = base case (WACC 8.58%, TGR 1.5%). Each TGR column uses its own growth path, fading to that rate by FY35. The WACC rows change discounting and terminal value only. Current price: €26.19.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -10716,9 +10717,10 @@
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B73" s="81" t="str">
-        <f aca="false">"Sensitivity, terminal growth "&amp;ROUND(DCF!$D$92*100,1)&amp;"%"</f>
-        <v>Sensitivity, terminal growth 0.5%</v>
+      <c r="B73" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sensitivity, terminal growth 0.5%</t>
+        </is>
       </c>
       <c r="C73" s="81"/>
       <c r="D73" s="81"/>
@@ -11307,9 +11309,10 @@
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B92" s="81" t="str">
-        <f aca="false">"Sensitivity, terminal growth "&amp;ROUND(DCF!$F$92*100,1)&amp;"%"</f>
-        <v>Sensitivity, terminal growth 1.0%</v>
+      <c r="B92" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sensitivity, terminal growth 1.0%</t>
+        </is>
       </c>
       <c r="C92" s="81"/>
       <c r="D92" s="81"/>
@@ -11898,9 +11901,10 @@
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B111" s="81" t="str">
-        <f aca="false">"Sensitivity, terminal growth "&amp;ROUND(DCF!$H$92*100,1)&amp;"%"</f>
-        <v>Sensitivity, terminal growth 1.5%</v>
+      <c r="B111" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sensitivity, terminal growth 1.5%</t>
+        </is>
       </c>
       <c r="C111" s="81"/>
       <c r="D111" s="81"/>
@@ -12489,9 +12493,10 @@
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B130" s="81" t="str">
-        <f aca="false">"Sensitivity, terminal growth "&amp;ROUND(DCF!$J$92*100,1)&amp;"%"</f>
-        <v>Sensitivity, terminal growth 2.0%</v>
+      <c r="B130" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sensitivity, terminal growth 2.0%</t>
+        </is>
       </c>
       <c r="C130" s="81"/>
       <c r="D130" s="81"/>
@@ -13080,9 +13085,10 @@
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B149" s="81" t="str">
-        <f aca="false">"Sensitivity, terminal growth "&amp;ROUND(DCF!$L$92*100,1)&amp;"%"</f>
-        <v>Sensitivity, terminal growth 2.5%</v>
+      <c r="B149" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sensitivity, terminal growth 2.5%</t>
+        </is>
       </c>
       <c r="C149" s="81"/>
       <c r="D149" s="81"/>

</xml_diff>